<commit_message>
ogrenci excel sablonu ve import sayfasi guncellendi
</commit_message>
<xml_diff>
--- a/public/ogrenci_sablonu.xlsx
+++ b/public/ogrenci_sablonu.xlsx
@@ -18,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -29,14 +29,19 @@
     <font>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
-      <sz val="11"/>
+      <sz val="10"/>
     </font>
     <font>
       <b val="1"/>
       <color rgb="001B4332"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <sz val="10"/>
     </font>
     <font>
       <color rgb="00000000"/>
+      <sz val="10"/>
     </font>
   </fonts>
   <fills count="4">
@@ -85,9 +90,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -98,6 +103,7 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -463,199 +469,288 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I204"/>
+  <dimension ref="A1:N204"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="15" customWidth="1" min="1" max="1"/>
+    <col width="6" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="20" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
-    <col width="15" customWidth="1" min="7" max="7"/>
-    <col width="16" customWidth="1" min="8" max="8"/>
-    <col width="20" customWidth="1" min="9" max="9"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="8" customWidth="1" min="7" max="7"/>
+    <col width="25" customWidth="1" min="8" max="8"/>
+    <col width="15" customWidth="1" min="9" max="9"/>
+    <col width="15" customWidth="1" min="10" max="10"/>
+    <col width="25" customWidth="1" min="11" max="11"/>
+    <col width="16" customWidth="1" min="12" max="12"/>
+    <col width="14" customWidth="1" min="13" max="13"/>
+    <col width="22" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
-    <row r="1" ht="35" customHeight="1">
+    <row r="1" ht="30" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Ad *</t>
+          <t>S.NO</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Soyad *</t>
+          <t>ADI *</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Doğum Tarihi (YYYY-AA-GG)</t>
+          <t>SOYADI *</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Cinsiyet (kiz/erkek) *</t>
+          <t>TC NO</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Veli Adı Soyadı *</t>
+          <t>DOĞUM TARİHİ</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Veli Telefonu *</t>
+          <t>CİNSİYET *</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>Mahalle</t>
+          <t>YAŞI</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>TC Kimlik No</t>
+          <t>ADRES</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>Sınıf Adı</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="20" customHeight="1">
-      <c r="A2" s="2" t="inlineStr">
+          <t>VELİ ADI *</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>VELİ SOYADI *</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>VELİ ADRESİ</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>GSM NUMARASI *</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>KAYIT TARİHİ</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>SINIF</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="18" customHeight="1">
+      <c r="A2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
         <is>
           <t>Ahmet</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="C2" s="2" t="inlineStr">
         <is>
           <t>Yılmaz</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>12345678901</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
         <is>
           <t>2015-03-15</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr">
+      <c r="F2" s="2" t="inlineStr">
         <is>
           <t>erkek</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>Mehmet Yılmaz</t>
-        </is>
-      </c>
-      <c r="F2" s="2" t="inlineStr">
+      <c r="G2" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>Havzan Mah. No:5</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>Mehmet</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>Yılmaz</t>
+        </is>
+      </c>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>Havzan Mah. No:5</t>
+        </is>
+      </c>
+      <c r="L2" s="2" t="inlineStr">
         <is>
           <t>05321234567</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr">
-        <is>
-          <t>Havzan</t>
-        </is>
-      </c>
-      <c r="H2" s="2" t="inlineStr">
-        <is>
-          <t>12345678901</t>
-        </is>
-      </c>
-      <c r="I2" s="2" t="inlineStr">
-        <is>
-          <t>Elif Sınıfı (7-8 Yaş Kızlar)</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="20" customHeight="1">
-      <c r="A3" s="2" t="inlineStr">
+      <c r="M2" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="N2" s="2" t="inlineStr">
+        <is>
+          <t>Elif Sınıfı</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="18" customHeight="1">
+      <c r="A3" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
         <is>
           <t>Fatma</t>
         </is>
       </c>
-      <c r="B3" s="2" t="inlineStr">
+      <c r="C3" s="2" t="inlineStr">
         <is>
           <t>Kaya</t>
         </is>
       </c>
-      <c r="C3" s="2" t="inlineStr">
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>98765432109</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
         <is>
           <t>2014-07-22</t>
         </is>
       </c>
-      <c r="D3" s="2" t="inlineStr">
+      <c r="F3" s="2" t="inlineStr">
         <is>
           <t>kiz</t>
         </is>
       </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>Ayşe Kaya</t>
-        </is>
-      </c>
-      <c r="F3" s="2" t="inlineStr">
+      <c r="G3" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>Karatay Mah. No:10</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>Ayşe</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>Kaya</t>
+        </is>
+      </c>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>Karatay Mah. No:10</t>
+        </is>
+      </c>
+      <c r="L3" s="2" t="inlineStr">
         <is>
           <t>05431234567</t>
         </is>
       </c>
-      <c r="G3" s="2" t="inlineStr">
-        <is>
-          <t>Karatay</t>
-        </is>
-      </c>
-      <c r="H3" s="2" t="inlineStr">
-        <is>
-          <t>98765432109</t>
-        </is>
-      </c>
-      <c r="I3" s="2" t="inlineStr">
-        <is>
-          <t>Havva Sınıfı (9-10 Yaş Kızlar)</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="20" customHeight="1">
-      <c r="A4" s="2" t="inlineStr">
+      <c r="M3" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="N3" s="2" t="inlineStr">
+        <is>
+          <t>Havva Sınıfı</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="18" customHeight="1">
+      <c r="A4" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
         <is>
           <t>Ali</t>
         </is>
       </c>
-      <c r="B4" s="2" t="inlineStr">
+      <c r="C4" s="2" t="inlineStr">
         <is>
           <t>Demir</t>
         </is>
       </c>
-      <c r="C4" s="2" t="inlineStr">
+      <c r="D4" s="2" t="inlineStr"/>
+      <c r="E4" s="2" t="inlineStr">
         <is>
           <t>2013-11-08</t>
         </is>
       </c>
-      <c r="D4" s="2" t="inlineStr">
+      <c r="F4" s="2" t="inlineStr">
         <is>
           <t>erkek</t>
         </is>
       </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>Hasan Demir</t>
-        </is>
-      </c>
-      <c r="F4" s="2" t="inlineStr">
+      <c r="G4" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>Selçuklu Mah.</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>Hasan</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>Demir</t>
+        </is>
+      </c>
+      <c r="K4" s="2" t="inlineStr"/>
+      <c r="L4" s="2" t="inlineStr">
         <is>
           <t>05531234567</t>
         </is>
       </c>
-      <c r="G4" s="2" t="inlineStr">
-        <is>
-          <t>Selçuklu</t>
-        </is>
-      </c>
-      <c r="H4" s="2" t="inlineStr"/>
-      <c r="I4" s="2" t="inlineStr"/>
+      <c r="M4" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="N4" s="2" t="inlineStr"/>
     </row>
     <row r="5" ht="18" customHeight="1">
       <c r="A5" s="3" t="inlineStr"/>
@@ -667,6 +762,11 @@
       <c r="G5" s="3" t="inlineStr"/>
       <c r="H5" s="3" t="inlineStr"/>
       <c r="I5" s="3" t="inlineStr"/>
+      <c r="J5" s="3" t="inlineStr"/>
+      <c r="K5" s="3" t="inlineStr"/>
+      <c r="L5" s="3" t="inlineStr"/>
+      <c r="M5" s="3" t="inlineStr"/>
+      <c r="N5" s="3" t="inlineStr"/>
     </row>
     <row r="6" ht="18" customHeight="1">
       <c r="A6" s="3" t="inlineStr"/>
@@ -678,6 +778,11 @@
       <c r="G6" s="3" t="inlineStr"/>
       <c r="H6" s="3" t="inlineStr"/>
       <c r="I6" s="3" t="inlineStr"/>
+      <c r="J6" s="3" t="inlineStr"/>
+      <c r="K6" s="3" t="inlineStr"/>
+      <c r="L6" s="3" t="inlineStr"/>
+      <c r="M6" s="3" t="inlineStr"/>
+      <c r="N6" s="3" t="inlineStr"/>
     </row>
     <row r="7" ht="18" customHeight="1">
       <c r="A7" s="3" t="inlineStr"/>
@@ -689,6 +794,11 @@
       <c r="G7" s="3" t="inlineStr"/>
       <c r="H7" s="3" t="inlineStr"/>
       <c r="I7" s="3" t="inlineStr"/>
+      <c r="J7" s="3" t="inlineStr"/>
+      <c r="K7" s="3" t="inlineStr"/>
+      <c r="L7" s="3" t="inlineStr"/>
+      <c r="M7" s="3" t="inlineStr"/>
+      <c r="N7" s="3" t="inlineStr"/>
     </row>
     <row r="8" ht="18" customHeight="1">
       <c r="A8" s="3" t="inlineStr"/>
@@ -700,6 +810,11 @@
       <c r="G8" s="3" t="inlineStr"/>
       <c r="H8" s="3" t="inlineStr"/>
       <c r="I8" s="3" t="inlineStr"/>
+      <c r="J8" s="3" t="inlineStr"/>
+      <c r="K8" s="3" t="inlineStr"/>
+      <c r="L8" s="3" t="inlineStr"/>
+      <c r="M8" s="3" t="inlineStr"/>
+      <c r="N8" s="3" t="inlineStr"/>
     </row>
     <row r="9" ht="18" customHeight="1">
       <c r="A9" s="3" t="inlineStr"/>
@@ -711,6 +826,11 @@
       <c r="G9" s="3" t="inlineStr"/>
       <c r="H9" s="3" t="inlineStr"/>
       <c r="I9" s="3" t="inlineStr"/>
+      <c r="J9" s="3" t="inlineStr"/>
+      <c r="K9" s="3" t="inlineStr"/>
+      <c r="L9" s="3" t="inlineStr"/>
+      <c r="M9" s="3" t="inlineStr"/>
+      <c r="N9" s="3" t="inlineStr"/>
     </row>
     <row r="10" ht="18" customHeight="1">
       <c r="A10" s="3" t="inlineStr"/>
@@ -722,6 +842,11 @@
       <c r="G10" s="3" t="inlineStr"/>
       <c r="H10" s="3" t="inlineStr"/>
       <c r="I10" s="3" t="inlineStr"/>
+      <c r="J10" s="3" t="inlineStr"/>
+      <c r="K10" s="3" t="inlineStr"/>
+      <c r="L10" s="3" t="inlineStr"/>
+      <c r="M10" s="3" t="inlineStr"/>
+      <c r="N10" s="3" t="inlineStr"/>
     </row>
     <row r="11" ht="18" customHeight="1">
       <c r="A11" s="3" t="inlineStr"/>
@@ -733,6 +858,11 @@
       <c r="G11" s="3" t="inlineStr"/>
       <c r="H11" s="3" t="inlineStr"/>
       <c r="I11" s="3" t="inlineStr"/>
+      <c r="J11" s="3" t="inlineStr"/>
+      <c r="K11" s="3" t="inlineStr"/>
+      <c r="L11" s="3" t="inlineStr"/>
+      <c r="M11" s="3" t="inlineStr"/>
+      <c r="N11" s="3" t="inlineStr"/>
     </row>
     <row r="12" ht="18" customHeight="1">
       <c r="A12" s="3" t="inlineStr"/>
@@ -744,6 +874,11 @@
       <c r="G12" s="3" t="inlineStr"/>
       <c r="H12" s="3" t="inlineStr"/>
       <c r="I12" s="3" t="inlineStr"/>
+      <c r="J12" s="3" t="inlineStr"/>
+      <c r="K12" s="3" t="inlineStr"/>
+      <c r="L12" s="3" t="inlineStr"/>
+      <c r="M12" s="3" t="inlineStr"/>
+      <c r="N12" s="3" t="inlineStr"/>
     </row>
     <row r="13" ht="18" customHeight="1">
       <c r="A13" s="3" t="inlineStr"/>
@@ -755,6 +890,11 @@
       <c r="G13" s="3" t="inlineStr"/>
       <c r="H13" s="3" t="inlineStr"/>
       <c r="I13" s="3" t="inlineStr"/>
+      <c r="J13" s="3" t="inlineStr"/>
+      <c r="K13" s="3" t="inlineStr"/>
+      <c r="L13" s="3" t="inlineStr"/>
+      <c r="M13" s="3" t="inlineStr"/>
+      <c r="N13" s="3" t="inlineStr"/>
     </row>
     <row r="14" ht="18" customHeight="1">
       <c r="A14" s="3" t="inlineStr"/>
@@ -766,6 +906,11 @@
       <c r="G14" s="3" t="inlineStr"/>
       <c r="H14" s="3" t="inlineStr"/>
       <c r="I14" s="3" t="inlineStr"/>
+      <c r="J14" s="3" t="inlineStr"/>
+      <c r="K14" s="3" t="inlineStr"/>
+      <c r="L14" s="3" t="inlineStr"/>
+      <c r="M14" s="3" t="inlineStr"/>
+      <c r="N14" s="3" t="inlineStr"/>
     </row>
     <row r="15" ht="18" customHeight="1">
       <c r="A15" s="3" t="inlineStr"/>
@@ -777,6 +922,11 @@
       <c r="G15" s="3" t="inlineStr"/>
       <c r="H15" s="3" t="inlineStr"/>
       <c r="I15" s="3" t="inlineStr"/>
+      <c r="J15" s="3" t="inlineStr"/>
+      <c r="K15" s="3" t="inlineStr"/>
+      <c r="L15" s="3" t="inlineStr"/>
+      <c r="M15" s="3" t="inlineStr"/>
+      <c r="N15" s="3" t="inlineStr"/>
     </row>
     <row r="16" ht="18" customHeight="1">
       <c r="A16" s="3" t="inlineStr"/>
@@ -788,6 +938,11 @@
       <c r="G16" s="3" t="inlineStr"/>
       <c r="H16" s="3" t="inlineStr"/>
       <c r="I16" s="3" t="inlineStr"/>
+      <c r="J16" s="3" t="inlineStr"/>
+      <c r="K16" s="3" t="inlineStr"/>
+      <c r="L16" s="3" t="inlineStr"/>
+      <c r="M16" s="3" t="inlineStr"/>
+      <c r="N16" s="3" t="inlineStr"/>
     </row>
     <row r="17" ht="18" customHeight="1">
       <c r="A17" s="3" t="inlineStr"/>
@@ -799,6 +954,11 @@
       <c r="G17" s="3" t="inlineStr"/>
       <c r="H17" s="3" t="inlineStr"/>
       <c r="I17" s="3" t="inlineStr"/>
+      <c r="J17" s="3" t="inlineStr"/>
+      <c r="K17" s="3" t="inlineStr"/>
+      <c r="L17" s="3" t="inlineStr"/>
+      <c r="M17" s="3" t="inlineStr"/>
+      <c r="N17" s="3" t="inlineStr"/>
     </row>
     <row r="18" ht="18" customHeight="1">
       <c r="A18" s="3" t="inlineStr"/>
@@ -810,6 +970,11 @@
       <c r="G18" s="3" t="inlineStr"/>
       <c r="H18" s="3" t="inlineStr"/>
       <c r="I18" s="3" t="inlineStr"/>
+      <c r="J18" s="3" t="inlineStr"/>
+      <c r="K18" s="3" t="inlineStr"/>
+      <c r="L18" s="3" t="inlineStr"/>
+      <c r="M18" s="3" t="inlineStr"/>
+      <c r="N18" s="3" t="inlineStr"/>
     </row>
     <row r="19" ht="18" customHeight="1">
       <c r="A19" s="3" t="inlineStr"/>
@@ -821,6 +986,11 @@
       <c r="G19" s="3" t="inlineStr"/>
       <c r="H19" s="3" t="inlineStr"/>
       <c r="I19" s="3" t="inlineStr"/>
+      <c r="J19" s="3" t="inlineStr"/>
+      <c r="K19" s="3" t="inlineStr"/>
+      <c r="L19" s="3" t="inlineStr"/>
+      <c r="M19" s="3" t="inlineStr"/>
+      <c r="N19" s="3" t="inlineStr"/>
     </row>
     <row r="20" ht="18" customHeight="1">
       <c r="A20" s="3" t="inlineStr"/>
@@ -832,6 +1002,11 @@
       <c r="G20" s="3" t="inlineStr"/>
       <c r="H20" s="3" t="inlineStr"/>
       <c r="I20" s="3" t="inlineStr"/>
+      <c r="J20" s="3" t="inlineStr"/>
+      <c r="K20" s="3" t="inlineStr"/>
+      <c r="L20" s="3" t="inlineStr"/>
+      <c r="M20" s="3" t="inlineStr"/>
+      <c r="N20" s="3" t="inlineStr"/>
     </row>
     <row r="21" ht="18" customHeight="1">
       <c r="A21" s="3" t="inlineStr"/>
@@ -843,6 +1018,11 @@
       <c r="G21" s="3" t="inlineStr"/>
       <c r="H21" s="3" t="inlineStr"/>
       <c r="I21" s="3" t="inlineStr"/>
+      <c r="J21" s="3" t="inlineStr"/>
+      <c r="K21" s="3" t="inlineStr"/>
+      <c r="L21" s="3" t="inlineStr"/>
+      <c r="M21" s="3" t="inlineStr"/>
+      <c r="N21" s="3" t="inlineStr"/>
     </row>
     <row r="22" ht="18" customHeight="1">
       <c r="A22" s="3" t="inlineStr"/>
@@ -854,6 +1034,11 @@
       <c r="G22" s="3" t="inlineStr"/>
       <c r="H22" s="3" t="inlineStr"/>
       <c r="I22" s="3" t="inlineStr"/>
+      <c r="J22" s="3" t="inlineStr"/>
+      <c r="K22" s="3" t="inlineStr"/>
+      <c r="L22" s="3" t="inlineStr"/>
+      <c r="M22" s="3" t="inlineStr"/>
+      <c r="N22" s="3" t="inlineStr"/>
     </row>
     <row r="23" ht="18" customHeight="1">
       <c r="A23" s="3" t="inlineStr"/>
@@ -865,6 +1050,11 @@
       <c r="G23" s="3" t="inlineStr"/>
       <c r="H23" s="3" t="inlineStr"/>
       <c r="I23" s="3" t="inlineStr"/>
+      <c r="J23" s="3" t="inlineStr"/>
+      <c r="K23" s="3" t="inlineStr"/>
+      <c r="L23" s="3" t="inlineStr"/>
+      <c r="M23" s="3" t="inlineStr"/>
+      <c r="N23" s="3" t="inlineStr"/>
     </row>
     <row r="24" ht="18" customHeight="1">
       <c r="A24" s="3" t="inlineStr"/>
@@ -876,6 +1066,11 @@
       <c r="G24" s="3" t="inlineStr"/>
       <c r="H24" s="3" t="inlineStr"/>
       <c r="I24" s="3" t="inlineStr"/>
+      <c r="J24" s="3" t="inlineStr"/>
+      <c r="K24" s="3" t="inlineStr"/>
+      <c r="L24" s="3" t="inlineStr"/>
+      <c r="M24" s="3" t="inlineStr"/>
+      <c r="N24" s="3" t="inlineStr"/>
     </row>
     <row r="25" ht="18" customHeight="1">
       <c r="A25" s="3" t="inlineStr"/>
@@ -887,6 +1082,11 @@
       <c r="G25" s="3" t="inlineStr"/>
       <c r="H25" s="3" t="inlineStr"/>
       <c r="I25" s="3" t="inlineStr"/>
+      <c r="J25" s="3" t="inlineStr"/>
+      <c r="K25" s="3" t="inlineStr"/>
+      <c r="L25" s="3" t="inlineStr"/>
+      <c r="M25" s="3" t="inlineStr"/>
+      <c r="N25" s="3" t="inlineStr"/>
     </row>
     <row r="26" ht="18" customHeight="1">
       <c r="A26" s="3" t="inlineStr"/>
@@ -898,6 +1098,11 @@
       <c r="G26" s="3" t="inlineStr"/>
       <c r="H26" s="3" t="inlineStr"/>
       <c r="I26" s="3" t="inlineStr"/>
+      <c r="J26" s="3" t="inlineStr"/>
+      <c r="K26" s="3" t="inlineStr"/>
+      <c r="L26" s="3" t="inlineStr"/>
+      <c r="M26" s="3" t="inlineStr"/>
+      <c r="N26" s="3" t="inlineStr"/>
     </row>
     <row r="27" ht="18" customHeight="1">
       <c r="A27" s="3" t="inlineStr"/>
@@ -909,6 +1114,11 @@
       <c r="G27" s="3" t="inlineStr"/>
       <c r="H27" s="3" t="inlineStr"/>
       <c r="I27" s="3" t="inlineStr"/>
+      <c r="J27" s="3" t="inlineStr"/>
+      <c r="K27" s="3" t="inlineStr"/>
+      <c r="L27" s="3" t="inlineStr"/>
+      <c r="M27" s="3" t="inlineStr"/>
+      <c r="N27" s="3" t="inlineStr"/>
     </row>
     <row r="28" ht="18" customHeight="1">
       <c r="A28" s="3" t="inlineStr"/>
@@ -920,6 +1130,11 @@
       <c r="G28" s="3" t="inlineStr"/>
       <c r="H28" s="3" t="inlineStr"/>
       <c r="I28" s="3" t="inlineStr"/>
+      <c r="J28" s="3" t="inlineStr"/>
+      <c r="K28" s="3" t="inlineStr"/>
+      <c r="L28" s="3" t="inlineStr"/>
+      <c r="M28" s="3" t="inlineStr"/>
+      <c r="N28" s="3" t="inlineStr"/>
     </row>
     <row r="29" ht="18" customHeight="1">
       <c r="A29" s="3" t="inlineStr"/>
@@ -931,6 +1146,11 @@
       <c r="G29" s="3" t="inlineStr"/>
       <c r="H29" s="3" t="inlineStr"/>
       <c r="I29" s="3" t="inlineStr"/>
+      <c r="J29" s="3" t="inlineStr"/>
+      <c r="K29" s="3" t="inlineStr"/>
+      <c r="L29" s="3" t="inlineStr"/>
+      <c r="M29" s="3" t="inlineStr"/>
+      <c r="N29" s="3" t="inlineStr"/>
     </row>
     <row r="30" ht="18" customHeight="1">
       <c r="A30" s="3" t="inlineStr"/>
@@ -942,6 +1162,11 @@
       <c r="G30" s="3" t="inlineStr"/>
       <c r="H30" s="3" t="inlineStr"/>
       <c r="I30" s="3" t="inlineStr"/>
+      <c r="J30" s="3" t="inlineStr"/>
+      <c r="K30" s="3" t="inlineStr"/>
+      <c r="L30" s="3" t="inlineStr"/>
+      <c r="M30" s="3" t="inlineStr"/>
+      <c r="N30" s="3" t="inlineStr"/>
     </row>
     <row r="31" ht="18" customHeight="1">
       <c r="A31" s="3" t="inlineStr"/>
@@ -953,6 +1178,11 @@
       <c r="G31" s="3" t="inlineStr"/>
       <c r="H31" s="3" t="inlineStr"/>
       <c r="I31" s="3" t="inlineStr"/>
+      <c r="J31" s="3" t="inlineStr"/>
+      <c r="K31" s="3" t="inlineStr"/>
+      <c r="L31" s="3" t="inlineStr"/>
+      <c r="M31" s="3" t="inlineStr"/>
+      <c r="N31" s="3" t="inlineStr"/>
     </row>
     <row r="32" ht="18" customHeight="1">
       <c r="A32" s="3" t="inlineStr"/>
@@ -964,6 +1194,11 @@
       <c r="G32" s="3" t="inlineStr"/>
       <c r="H32" s="3" t="inlineStr"/>
       <c r="I32" s="3" t="inlineStr"/>
+      <c r="J32" s="3" t="inlineStr"/>
+      <c r="K32" s="3" t="inlineStr"/>
+      <c r="L32" s="3" t="inlineStr"/>
+      <c r="M32" s="3" t="inlineStr"/>
+      <c r="N32" s="3" t="inlineStr"/>
     </row>
     <row r="33" ht="18" customHeight="1">
       <c r="A33" s="3" t="inlineStr"/>
@@ -975,6 +1210,11 @@
       <c r="G33" s="3" t="inlineStr"/>
       <c r="H33" s="3" t="inlineStr"/>
       <c r="I33" s="3" t="inlineStr"/>
+      <c r="J33" s="3" t="inlineStr"/>
+      <c r="K33" s="3" t="inlineStr"/>
+      <c r="L33" s="3" t="inlineStr"/>
+      <c r="M33" s="3" t="inlineStr"/>
+      <c r="N33" s="3" t="inlineStr"/>
     </row>
     <row r="34" ht="18" customHeight="1">
       <c r="A34" s="3" t="inlineStr"/>
@@ -986,6 +1226,11 @@
       <c r="G34" s="3" t="inlineStr"/>
       <c r="H34" s="3" t="inlineStr"/>
       <c r="I34" s="3" t="inlineStr"/>
+      <c r="J34" s="3" t="inlineStr"/>
+      <c r="K34" s="3" t="inlineStr"/>
+      <c r="L34" s="3" t="inlineStr"/>
+      <c r="M34" s="3" t="inlineStr"/>
+      <c r="N34" s="3" t="inlineStr"/>
     </row>
     <row r="35" ht="18" customHeight="1">
       <c r="A35" s="3" t="inlineStr"/>
@@ -997,6 +1242,11 @@
       <c r="G35" s="3" t="inlineStr"/>
       <c r="H35" s="3" t="inlineStr"/>
       <c r="I35" s="3" t="inlineStr"/>
+      <c r="J35" s="3" t="inlineStr"/>
+      <c r="K35" s="3" t="inlineStr"/>
+      <c r="L35" s="3" t="inlineStr"/>
+      <c r="M35" s="3" t="inlineStr"/>
+      <c r="N35" s="3" t="inlineStr"/>
     </row>
     <row r="36" ht="18" customHeight="1">
       <c r="A36" s="3" t="inlineStr"/>
@@ -1008,6 +1258,11 @@
       <c r="G36" s="3" t="inlineStr"/>
       <c r="H36" s="3" t="inlineStr"/>
       <c r="I36" s="3" t="inlineStr"/>
+      <c r="J36" s="3" t="inlineStr"/>
+      <c r="K36" s="3" t="inlineStr"/>
+      <c r="L36" s="3" t="inlineStr"/>
+      <c r="M36" s="3" t="inlineStr"/>
+      <c r="N36" s="3" t="inlineStr"/>
     </row>
     <row r="37" ht="18" customHeight="1">
       <c r="A37" s="3" t="inlineStr"/>
@@ -1019,6 +1274,11 @@
       <c r="G37" s="3" t="inlineStr"/>
       <c r="H37" s="3" t="inlineStr"/>
       <c r="I37" s="3" t="inlineStr"/>
+      <c r="J37" s="3" t="inlineStr"/>
+      <c r="K37" s="3" t="inlineStr"/>
+      <c r="L37" s="3" t="inlineStr"/>
+      <c r="M37" s="3" t="inlineStr"/>
+      <c r="N37" s="3" t="inlineStr"/>
     </row>
     <row r="38" ht="18" customHeight="1">
       <c r="A38" s="3" t="inlineStr"/>
@@ -1030,6 +1290,11 @@
       <c r="G38" s="3" t="inlineStr"/>
       <c r="H38" s="3" t="inlineStr"/>
       <c r="I38" s="3" t="inlineStr"/>
+      <c r="J38" s="3" t="inlineStr"/>
+      <c r="K38" s="3" t="inlineStr"/>
+      <c r="L38" s="3" t="inlineStr"/>
+      <c r="M38" s="3" t="inlineStr"/>
+      <c r="N38" s="3" t="inlineStr"/>
     </row>
     <row r="39" ht="18" customHeight="1">
       <c r="A39" s="3" t="inlineStr"/>
@@ -1041,6 +1306,11 @@
       <c r="G39" s="3" t="inlineStr"/>
       <c r="H39" s="3" t="inlineStr"/>
       <c r="I39" s="3" t="inlineStr"/>
+      <c r="J39" s="3" t="inlineStr"/>
+      <c r="K39" s="3" t="inlineStr"/>
+      <c r="L39" s="3" t="inlineStr"/>
+      <c r="M39" s="3" t="inlineStr"/>
+      <c r="N39" s="3" t="inlineStr"/>
     </row>
     <row r="40" ht="18" customHeight="1">
       <c r="A40" s="3" t="inlineStr"/>
@@ -1052,6 +1322,11 @@
       <c r="G40" s="3" t="inlineStr"/>
       <c r="H40" s="3" t="inlineStr"/>
       <c r="I40" s="3" t="inlineStr"/>
+      <c r="J40" s="3" t="inlineStr"/>
+      <c r="K40" s="3" t="inlineStr"/>
+      <c r="L40" s="3" t="inlineStr"/>
+      <c r="M40" s="3" t="inlineStr"/>
+      <c r="N40" s="3" t="inlineStr"/>
     </row>
     <row r="41" ht="18" customHeight="1">
       <c r="A41" s="3" t="inlineStr"/>
@@ -1063,6 +1338,11 @@
       <c r="G41" s="3" t="inlineStr"/>
       <c r="H41" s="3" t="inlineStr"/>
       <c r="I41" s="3" t="inlineStr"/>
+      <c r="J41" s="3" t="inlineStr"/>
+      <c r="K41" s="3" t="inlineStr"/>
+      <c r="L41" s="3" t="inlineStr"/>
+      <c r="M41" s="3" t="inlineStr"/>
+      <c r="N41" s="3" t="inlineStr"/>
     </row>
     <row r="42" ht="18" customHeight="1">
       <c r="A42" s="3" t="inlineStr"/>
@@ -1074,6 +1354,11 @@
       <c r="G42" s="3" t="inlineStr"/>
       <c r="H42" s="3" t="inlineStr"/>
       <c r="I42" s="3" t="inlineStr"/>
+      <c r="J42" s="3" t="inlineStr"/>
+      <c r="K42" s="3" t="inlineStr"/>
+      <c r="L42" s="3" t="inlineStr"/>
+      <c r="M42" s="3" t="inlineStr"/>
+      <c r="N42" s="3" t="inlineStr"/>
     </row>
     <row r="43" ht="18" customHeight="1">
       <c r="A43" s="3" t="inlineStr"/>
@@ -1085,6 +1370,11 @@
       <c r="G43" s="3" t="inlineStr"/>
       <c r="H43" s="3" t="inlineStr"/>
       <c r="I43" s="3" t="inlineStr"/>
+      <c r="J43" s="3" t="inlineStr"/>
+      <c r="K43" s="3" t="inlineStr"/>
+      <c r="L43" s="3" t="inlineStr"/>
+      <c r="M43" s="3" t="inlineStr"/>
+      <c r="N43" s="3" t="inlineStr"/>
     </row>
     <row r="44" ht="18" customHeight="1">
       <c r="A44" s="3" t="inlineStr"/>
@@ -1096,6 +1386,11 @@
       <c r="G44" s="3" t="inlineStr"/>
       <c r="H44" s="3" t="inlineStr"/>
       <c r="I44" s="3" t="inlineStr"/>
+      <c r="J44" s="3" t="inlineStr"/>
+      <c r="K44" s="3" t="inlineStr"/>
+      <c r="L44" s="3" t="inlineStr"/>
+      <c r="M44" s="3" t="inlineStr"/>
+      <c r="N44" s="3" t="inlineStr"/>
     </row>
     <row r="45" ht="18" customHeight="1">
       <c r="A45" s="3" t="inlineStr"/>
@@ -1107,6 +1402,11 @@
       <c r="G45" s="3" t="inlineStr"/>
       <c r="H45" s="3" t="inlineStr"/>
       <c r="I45" s="3" t="inlineStr"/>
+      <c r="J45" s="3" t="inlineStr"/>
+      <c r="K45" s="3" t="inlineStr"/>
+      <c r="L45" s="3" t="inlineStr"/>
+      <c r="M45" s="3" t="inlineStr"/>
+      <c r="N45" s="3" t="inlineStr"/>
     </row>
     <row r="46" ht="18" customHeight="1">
       <c r="A46" s="3" t="inlineStr"/>
@@ -1118,6 +1418,11 @@
       <c r="G46" s="3" t="inlineStr"/>
       <c r="H46" s="3" t="inlineStr"/>
       <c r="I46" s="3" t="inlineStr"/>
+      <c r="J46" s="3" t="inlineStr"/>
+      <c r="K46" s="3" t="inlineStr"/>
+      <c r="L46" s="3" t="inlineStr"/>
+      <c r="M46" s="3" t="inlineStr"/>
+      <c r="N46" s="3" t="inlineStr"/>
     </row>
     <row r="47" ht="18" customHeight="1">
       <c r="A47" s="3" t="inlineStr"/>
@@ -1129,6 +1434,11 @@
       <c r="G47" s="3" t="inlineStr"/>
       <c r="H47" s="3" t="inlineStr"/>
       <c r="I47" s="3" t="inlineStr"/>
+      <c r="J47" s="3" t="inlineStr"/>
+      <c r="K47" s="3" t="inlineStr"/>
+      <c r="L47" s="3" t="inlineStr"/>
+      <c r="M47" s="3" t="inlineStr"/>
+      <c r="N47" s="3" t="inlineStr"/>
     </row>
     <row r="48" ht="18" customHeight="1">
       <c r="A48" s="3" t="inlineStr"/>
@@ -1140,6 +1450,11 @@
       <c r="G48" s="3" t="inlineStr"/>
       <c r="H48" s="3" t="inlineStr"/>
       <c r="I48" s="3" t="inlineStr"/>
+      <c r="J48" s="3" t="inlineStr"/>
+      <c r="K48" s="3" t="inlineStr"/>
+      <c r="L48" s="3" t="inlineStr"/>
+      <c r="M48" s="3" t="inlineStr"/>
+      <c r="N48" s="3" t="inlineStr"/>
     </row>
     <row r="49" ht="18" customHeight="1">
       <c r="A49" s="3" t="inlineStr"/>
@@ -1151,6 +1466,11 @@
       <c r="G49" s="3" t="inlineStr"/>
       <c r="H49" s="3" t="inlineStr"/>
       <c r="I49" s="3" t="inlineStr"/>
+      <c r="J49" s="3" t="inlineStr"/>
+      <c r="K49" s="3" t="inlineStr"/>
+      <c r="L49" s="3" t="inlineStr"/>
+      <c r="M49" s="3" t="inlineStr"/>
+      <c r="N49" s="3" t="inlineStr"/>
     </row>
     <row r="50" ht="18" customHeight="1">
       <c r="A50" s="3" t="inlineStr"/>
@@ -1162,6 +1482,11 @@
       <c r="G50" s="3" t="inlineStr"/>
       <c r="H50" s="3" t="inlineStr"/>
       <c r="I50" s="3" t="inlineStr"/>
+      <c r="J50" s="3" t="inlineStr"/>
+      <c r="K50" s="3" t="inlineStr"/>
+      <c r="L50" s="3" t="inlineStr"/>
+      <c r="M50" s="3" t="inlineStr"/>
+      <c r="N50" s="3" t="inlineStr"/>
     </row>
     <row r="51" ht="18" customHeight="1">
       <c r="A51" s="3" t="inlineStr"/>
@@ -1173,6 +1498,11 @@
       <c r="G51" s="3" t="inlineStr"/>
       <c r="H51" s="3" t="inlineStr"/>
       <c r="I51" s="3" t="inlineStr"/>
+      <c r="J51" s="3" t="inlineStr"/>
+      <c r="K51" s="3" t="inlineStr"/>
+      <c r="L51" s="3" t="inlineStr"/>
+      <c r="M51" s="3" t="inlineStr"/>
+      <c r="N51" s="3" t="inlineStr"/>
     </row>
     <row r="52" ht="18" customHeight="1">
       <c r="A52" s="3" t="inlineStr"/>
@@ -1184,6 +1514,11 @@
       <c r="G52" s="3" t="inlineStr"/>
       <c r="H52" s="3" t="inlineStr"/>
       <c r="I52" s="3" t="inlineStr"/>
+      <c r="J52" s="3" t="inlineStr"/>
+      <c r="K52" s="3" t="inlineStr"/>
+      <c r="L52" s="3" t="inlineStr"/>
+      <c r="M52" s="3" t="inlineStr"/>
+      <c r="N52" s="3" t="inlineStr"/>
     </row>
     <row r="53" ht="18" customHeight="1">
       <c r="A53" s="3" t="inlineStr"/>
@@ -1195,6 +1530,11 @@
       <c r="G53" s="3" t="inlineStr"/>
       <c r="H53" s="3" t="inlineStr"/>
       <c r="I53" s="3" t="inlineStr"/>
+      <c r="J53" s="3" t="inlineStr"/>
+      <c r="K53" s="3" t="inlineStr"/>
+      <c r="L53" s="3" t="inlineStr"/>
+      <c r="M53" s="3" t="inlineStr"/>
+      <c r="N53" s="3" t="inlineStr"/>
     </row>
     <row r="54" ht="18" customHeight="1">
       <c r="A54" s="3" t="inlineStr"/>
@@ -1206,6 +1546,11 @@
       <c r="G54" s="3" t="inlineStr"/>
       <c r="H54" s="3" t="inlineStr"/>
       <c r="I54" s="3" t="inlineStr"/>
+      <c r="J54" s="3" t="inlineStr"/>
+      <c r="K54" s="3" t="inlineStr"/>
+      <c r="L54" s="3" t="inlineStr"/>
+      <c r="M54" s="3" t="inlineStr"/>
+      <c r="N54" s="3" t="inlineStr"/>
     </row>
     <row r="55" ht="18" customHeight="1">
       <c r="A55" s="3" t="inlineStr"/>
@@ -1217,6 +1562,11 @@
       <c r="G55" s="3" t="inlineStr"/>
       <c r="H55" s="3" t="inlineStr"/>
       <c r="I55" s="3" t="inlineStr"/>
+      <c r="J55" s="3" t="inlineStr"/>
+      <c r="K55" s="3" t="inlineStr"/>
+      <c r="L55" s="3" t="inlineStr"/>
+      <c r="M55" s="3" t="inlineStr"/>
+      <c r="N55" s="3" t="inlineStr"/>
     </row>
     <row r="56" ht="18" customHeight="1">
       <c r="A56" s="3" t="inlineStr"/>
@@ -1228,6 +1578,11 @@
       <c r="G56" s="3" t="inlineStr"/>
       <c r="H56" s="3" t="inlineStr"/>
       <c r="I56" s="3" t="inlineStr"/>
+      <c r="J56" s="3" t="inlineStr"/>
+      <c r="K56" s="3" t="inlineStr"/>
+      <c r="L56" s="3" t="inlineStr"/>
+      <c r="M56" s="3" t="inlineStr"/>
+      <c r="N56" s="3" t="inlineStr"/>
     </row>
     <row r="57" ht="18" customHeight="1">
       <c r="A57" s="3" t="inlineStr"/>
@@ -1239,6 +1594,11 @@
       <c r="G57" s="3" t="inlineStr"/>
       <c r="H57" s="3" t="inlineStr"/>
       <c r="I57" s="3" t="inlineStr"/>
+      <c r="J57" s="3" t="inlineStr"/>
+      <c r="K57" s="3" t="inlineStr"/>
+      <c r="L57" s="3" t="inlineStr"/>
+      <c r="M57" s="3" t="inlineStr"/>
+      <c r="N57" s="3" t="inlineStr"/>
     </row>
     <row r="58" ht="18" customHeight="1">
       <c r="A58" s="3" t="inlineStr"/>
@@ -1250,6 +1610,11 @@
       <c r="G58" s="3" t="inlineStr"/>
       <c r="H58" s="3" t="inlineStr"/>
       <c r="I58" s="3" t="inlineStr"/>
+      <c r="J58" s="3" t="inlineStr"/>
+      <c r="K58" s="3" t="inlineStr"/>
+      <c r="L58" s="3" t="inlineStr"/>
+      <c r="M58" s="3" t="inlineStr"/>
+      <c r="N58" s="3" t="inlineStr"/>
     </row>
     <row r="59" ht="18" customHeight="1">
       <c r="A59" s="3" t="inlineStr"/>
@@ -1261,6 +1626,11 @@
       <c r="G59" s="3" t="inlineStr"/>
       <c r="H59" s="3" t="inlineStr"/>
       <c r="I59" s="3" t="inlineStr"/>
+      <c r="J59" s="3" t="inlineStr"/>
+      <c r="K59" s="3" t="inlineStr"/>
+      <c r="L59" s="3" t="inlineStr"/>
+      <c r="M59" s="3" t="inlineStr"/>
+      <c r="N59" s="3" t="inlineStr"/>
     </row>
     <row r="60" ht="18" customHeight="1">
       <c r="A60" s="3" t="inlineStr"/>
@@ -1272,6 +1642,11 @@
       <c r="G60" s="3" t="inlineStr"/>
       <c r="H60" s="3" t="inlineStr"/>
       <c r="I60" s="3" t="inlineStr"/>
+      <c r="J60" s="3" t="inlineStr"/>
+      <c r="K60" s="3" t="inlineStr"/>
+      <c r="L60" s="3" t="inlineStr"/>
+      <c r="M60" s="3" t="inlineStr"/>
+      <c r="N60" s="3" t="inlineStr"/>
     </row>
     <row r="61" ht="18" customHeight="1">
       <c r="A61" s="3" t="inlineStr"/>
@@ -1283,6 +1658,11 @@
       <c r="G61" s="3" t="inlineStr"/>
       <c r="H61" s="3" t="inlineStr"/>
       <c r="I61" s="3" t="inlineStr"/>
+      <c r="J61" s="3" t="inlineStr"/>
+      <c r="K61" s="3" t="inlineStr"/>
+      <c r="L61" s="3" t="inlineStr"/>
+      <c r="M61" s="3" t="inlineStr"/>
+      <c r="N61" s="3" t="inlineStr"/>
     </row>
     <row r="62" ht="18" customHeight="1">
       <c r="A62" s="3" t="inlineStr"/>
@@ -1294,6 +1674,11 @@
       <c r="G62" s="3" t="inlineStr"/>
       <c r="H62" s="3" t="inlineStr"/>
       <c r="I62" s="3" t="inlineStr"/>
+      <c r="J62" s="3" t="inlineStr"/>
+      <c r="K62" s="3" t="inlineStr"/>
+      <c r="L62" s="3" t="inlineStr"/>
+      <c r="M62" s="3" t="inlineStr"/>
+      <c r="N62" s="3" t="inlineStr"/>
     </row>
     <row r="63" ht="18" customHeight="1">
       <c r="A63" s="3" t="inlineStr"/>
@@ -1305,6 +1690,11 @@
       <c r="G63" s="3" t="inlineStr"/>
       <c r="H63" s="3" t="inlineStr"/>
       <c r="I63" s="3" t="inlineStr"/>
+      <c r="J63" s="3" t="inlineStr"/>
+      <c r="K63" s="3" t="inlineStr"/>
+      <c r="L63" s="3" t="inlineStr"/>
+      <c r="M63" s="3" t="inlineStr"/>
+      <c r="N63" s="3" t="inlineStr"/>
     </row>
     <row r="64" ht="18" customHeight="1">
       <c r="A64" s="3" t="inlineStr"/>
@@ -1316,6 +1706,11 @@
       <c r="G64" s="3" t="inlineStr"/>
       <c r="H64" s="3" t="inlineStr"/>
       <c r="I64" s="3" t="inlineStr"/>
+      <c r="J64" s="3" t="inlineStr"/>
+      <c r="K64" s="3" t="inlineStr"/>
+      <c r="L64" s="3" t="inlineStr"/>
+      <c r="M64" s="3" t="inlineStr"/>
+      <c r="N64" s="3" t="inlineStr"/>
     </row>
     <row r="65" ht="18" customHeight="1">
       <c r="A65" s="3" t="inlineStr"/>
@@ -1327,6 +1722,11 @@
       <c r="G65" s="3" t="inlineStr"/>
       <c r="H65" s="3" t="inlineStr"/>
       <c r="I65" s="3" t="inlineStr"/>
+      <c r="J65" s="3" t="inlineStr"/>
+      <c r="K65" s="3" t="inlineStr"/>
+      <c r="L65" s="3" t="inlineStr"/>
+      <c r="M65" s="3" t="inlineStr"/>
+      <c r="N65" s="3" t="inlineStr"/>
     </row>
     <row r="66" ht="18" customHeight="1">
       <c r="A66" s="3" t="inlineStr"/>
@@ -1338,6 +1738,11 @@
       <c r="G66" s="3" t="inlineStr"/>
       <c r="H66" s="3" t="inlineStr"/>
       <c r="I66" s="3" t="inlineStr"/>
+      <c r="J66" s="3" t="inlineStr"/>
+      <c r="K66" s="3" t="inlineStr"/>
+      <c r="L66" s="3" t="inlineStr"/>
+      <c r="M66" s="3" t="inlineStr"/>
+      <c r="N66" s="3" t="inlineStr"/>
     </row>
     <row r="67" ht="18" customHeight="1">
       <c r="A67" s="3" t="inlineStr"/>
@@ -1349,6 +1754,11 @@
       <c r="G67" s="3" t="inlineStr"/>
       <c r="H67" s="3" t="inlineStr"/>
       <c r="I67" s="3" t="inlineStr"/>
+      <c r="J67" s="3" t="inlineStr"/>
+      <c r="K67" s="3" t="inlineStr"/>
+      <c r="L67" s="3" t="inlineStr"/>
+      <c r="M67" s="3" t="inlineStr"/>
+      <c r="N67" s="3" t="inlineStr"/>
     </row>
     <row r="68" ht="18" customHeight="1">
       <c r="A68" s="3" t="inlineStr"/>
@@ -1360,6 +1770,11 @@
       <c r="G68" s="3" t="inlineStr"/>
       <c r="H68" s="3" t="inlineStr"/>
       <c r="I68" s="3" t="inlineStr"/>
+      <c r="J68" s="3" t="inlineStr"/>
+      <c r="K68" s="3" t="inlineStr"/>
+      <c r="L68" s="3" t="inlineStr"/>
+      <c r="M68" s="3" t="inlineStr"/>
+      <c r="N68" s="3" t="inlineStr"/>
     </row>
     <row r="69" ht="18" customHeight="1">
       <c r="A69" s="3" t="inlineStr"/>
@@ -1371,6 +1786,11 @@
       <c r="G69" s="3" t="inlineStr"/>
       <c r="H69" s="3" t="inlineStr"/>
       <c r="I69" s="3" t="inlineStr"/>
+      <c r="J69" s="3" t="inlineStr"/>
+      <c r="K69" s="3" t="inlineStr"/>
+      <c r="L69" s="3" t="inlineStr"/>
+      <c r="M69" s="3" t="inlineStr"/>
+      <c r="N69" s="3" t="inlineStr"/>
     </row>
     <row r="70" ht="18" customHeight="1">
       <c r="A70" s="3" t="inlineStr"/>
@@ -1382,6 +1802,11 @@
       <c r="G70" s="3" t="inlineStr"/>
       <c r="H70" s="3" t="inlineStr"/>
       <c r="I70" s="3" t="inlineStr"/>
+      <c r="J70" s="3" t="inlineStr"/>
+      <c r="K70" s="3" t="inlineStr"/>
+      <c r="L70" s="3" t="inlineStr"/>
+      <c r="M70" s="3" t="inlineStr"/>
+      <c r="N70" s="3" t="inlineStr"/>
     </row>
     <row r="71" ht="18" customHeight="1">
       <c r="A71" s="3" t="inlineStr"/>
@@ -1393,6 +1818,11 @@
       <c r="G71" s="3" t="inlineStr"/>
       <c r="H71" s="3" t="inlineStr"/>
       <c r="I71" s="3" t="inlineStr"/>
+      <c r="J71" s="3" t="inlineStr"/>
+      <c r="K71" s="3" t="inlineStr"/>
+      <c r="L71" s="3" t="inlineStr"/>
+      <c r="M71" s="3" t="inlineStr"/>
+      <c r="N71" s="3" t="inlineStr"/>
     </row>
     <row r="72" ht="18" customHeight="1">
       <c r="A72" s="3" t="inlineStr"/>
@@ -1404,6 +1834,11 @@
       <c r="G72" s="3" t="inlineStr"/>
       <c r="H72" s="3" t="inlineStr"/>
       <c r="I72" s="3" t="inlineStr"/>
+      <c r="J72" s="3" t="inlineStr"/>
+      <c r="K72" s="3" t="inlineStr"/>
+      <c r="L72" s="3" t="inlineStr"/>
+      <c r="M72" s="3" t="inlineStr"/>
+      <c r="N72" s="3" t="inlineStr"/>
     </row>
     <row r="73" ht="18" customHeight="1">
       <c r="A73" s="3" t="inlineStr"/>
@@ -1415,6 +1850,11 @@
       <c r="G73" s="3" t="inlineStr"/>
       <c r="H73" s="3" t="inlineStr"/>
       <c r="I73" s="3" t="inlineStr"/>
+      <c r="J73" s="3" t="inlineStr"/>
+      <c r="K73" s="3" t="inlineStr"/>
+      <c r="L73" s="3" t="inlineStr"/>
+      <c r="M73" s="3" t="inlineStr"/>
+      <c r="N73" s="3" t="inlineStr"/>
     </row>
     <row r="74" ht="18" customHeight="1">
       <c r="A74" s="3" t="inlineStr"/>
@@ -1426,6 +1866,11 @@
       <c r="G74" s="3" t="inlineStr"/>
       <c r="H74" s="3" t="inlineStr"/>
       <c r="I74" s="3" t="inlineStr"/>
+      <c r="J74" s="3" t="inlineStr"/>
+      <c r="K74" s="3" t="inlineStr"/>
+      <c r="L74" s="3" t="inlineStr"/>
+      <c r="M74" s="3" t="inlineStr"/>
+      <c r="N74" s="3" t="inlineStr"/>
     </row>
     <row r="75" ht="18" customHeight="1">
       <c r="A75" s="3" t="inlineStr"/>
@@ -1437,6 +1882,11 @@
       <c r="G75" s="3" t="inlineStr"/>
       <c r="H75" s="3" t="inlineStr"/>
       <c r="I75" s="3" t="inlineStr"/>
+      <c r="J75" s="3" t="inlineStr"/>
+      <c r="K75" s="3" t="inlineStr"/>
+      <c r="L75" s="3" t="inlineStr"/>
+      <c r="M75" s="3" t="inlineStr"/>
+      <c r="N75" s="3" t="inlineStr"/>
     </row>
     <row r="76" ht="18" customHeight="1">
       <c r="A76" s="3" t="inlineStr"/>
@@ -1448,6 +1898,11 @@
       <c r="G76" s="3" t="inlineStr"/>
       <c r="H76" s="3" t="inlineStr"/>
       <c r="I76" s="3" t="inlineStr"/>
+      <c r="J76" s="3" t="inlineStr"/>
+      <c r="K76" s="3" t="inlineStr"/>
+      <c r="L76" s="3" t="inlineStr"/>
+      <c r="M76" s="3" t="inlineStr"/>
+      <c r="N76" s="3" t="inlineStr"/>
     </row>
     <row r="77" ht="18" customHeight="1">
       <c r="A77" s="3" t="inlineStr"/>
@@ -1459,6 +1914,11 @@
       <c r="G77" s="3" t="inlineStr"/>
       <c r="H77" s="3" t="inlineStr"/>
       <c r="I77" s="3" t="inlineStr"/>
+      <c r="J77" s="3" t="inlineStr"/>
+      <c r="K77" s="3" t="inlineStr"/>
+      <c r="L77" s="3" t="inlineStr"/>
+      <c r="M77" s="3" t="inlineStr"/>
+      <c r="N77" s="3" t="inlineStr"/>
     </row>
     <row r="78" ht="18" customHeight="1">
       <c r="A78" s="3" t="inlineStr"/>
@@ -1470,6 +1930,11 @@
       <c r="G78" s="3" t="inlineStr"/>
       <c r="H78" s="3" t="inlineStr"/>
       <c r="I78" s="3" t="inlineStr"/>
+      <c r="J78" s="3" t="inlineStr"/>
+      <c r="K78" s="3" t="inlineStr"/>
+      <c r="L78" s="3" t="inlineStr"/>
+      <c r="M78" s="3" t="inlineStr"/>
+      <c r="N78" s="3" t="inlineStr"/>
     </row>
     <row r="79" ht="18" customHeight="1">
       <c r="A79" s="3" t="inlineStr"/>
@@ -1481,6 +1946,11 @@
       <c r="G79" s="3" t="inlineStr"/>
       <c r="H79" s="3" t="inlineStr"/>
       <c r="I79" s="3" t="inlineStr"/>
+      <c r="J79" s="3" t="inlineStr"/>
+      <c r="K79" s="3" t="inlineStr"/>
+      <c r="L79" s="3" t="inlineStr"/>
+      <c r="M79" s="3" t="inlineStr"/>
+      <c r="N79" s="3" t="inlineStr"/>
     </row>
     <row r="80" ht="18" customHeight="1">
       <c r="A80" s="3" t="inlineStr"/>
@@ -1492,6 +1962,11 @@
       <c r="G80" s="3" t="inlineStr"/>
       <c r="H80" s="3" t="inlineStr"/>
       <c r="I80" s="3" t="inlineStr"/>
+      <c r="J80" s="3" t="inlineStr"/>
+      <c r="K80" s="3" t="inlineStr"/>
+      <c r="L80" s="3" t="inlineStr"/>
+      <c r="M80" s="3" t="inlineStr"/>
+      <c r="N80" s="3" t="inlineStr"/>
     </row>
     <row r="81" ht="18" customHeight="1">
       <c r="A81" s="3" t="inlineStr"/>
@@ -1503,6 +1978,11 @@
       <c r="G81" s="3" t="inlineStr"/>
       <c r="H81" s="3" t="inlineStr"/>
       <c r="I81" s="3" t="inlineStr"/>
+      <c r="J81" s="3" t="inlineStr"/>
+      <c r="K81" s="3" t="inlineStr"/>
+      <c r="L81" s="3" t="inlineStr"/>
+      <c r="M81" s="3" t="inlineStr"/>
+      <c r="N81" s="3" t="inlineStr"/>
     </row>
     <row r="82" ht="18" customHeight="1">
       <c r="A82" s="3" t="inlineStr"/>
@@ -1514,6 +1994,11 @@
       <c r="G82" s="3" t="inlineStr"/>
       <c r="H82" s="3" t="inlineStr"/>
       <c r="I82" s="3" t="inlineStr"/>
+      <c r="J82" s="3" t="inlineStr"/>
+      <c r="K82" s="3" t="inlineStr"/>
+      <c r="L82" s="3" t="inlineStr"/>
+      <c r="M82" s="3" t="inlineStr"/>
+      <c r="N82" s="3" t="inlineStr"/>
     </row>
     <row r="83" ht="18" customHeight="1">
       <c r="A83" s="3" t="inlineStr"/>
@@ -1525,6 +2010,11 @@
       <c r="G83" s="3" t="inlineStr"/>
       <c r="H83" s="3" t="inlineStr"/>
       <c r="I83" s="3" t="inlineStr"/>
+      <c r="J83" s="3" t="inlineStr"/>
+      <c r="K83" s="3" t="inlineStr"/>
+      <c r="L83" s="3" t="inlineStr"/>
+      <c r="M83" s="3" t="inlineStr"/>
+      <c r="N83" s="3" t="inlineStr"/>
     </row>
     <row r="84" ht="18" customHeight="1">
       <c r="A84" s="3" t="inlineStr"/>
@@ -1536,6 +2026,11 @@
       <c r="G84" s="3" t="inlineStr"/>
       <c r="H84" s="3" t="inlineStr"/>
       <c r="I84" s="3" t="inlineStr"/>
+      <c r="J84" s="3" t="inlineStr"/>
+      <c r="K84" s="3" t="inlineStr"/>
+      <c r="L84" s="3" t="inlineStr"/>
+      <c r="M84" s="3" t="inlineStr"/>
+      <c r="N84" s="3" t="inlineStr"/>
     </row>
     <row r="85" ht="18" customHeight="1">
       <c r="A85" s="3" t="inlineStr"/>
@@ -1547,6 +2042,11 @@
       <c r="G85" s="3" t="inlineStr"/>
       <c r="H85" s="3" t="inlineStr"/>
       <c r="I85" s="3" t="inlineStr"/>
+      <c r="J85" s="3" t="inlineStr"/>
+      <c r="K85" s="3" t="inlineStr"/>
+      <c r="L85" s="3" t="inlineStr"/>
+      <c r="M85" s="3" t="inlineStr"/>
+      <c r="N85" s="3" t="inlineStr"/>
     </row>
     <row r="86" ht="18" customHeight="1">
       <c r="A86" s="3" t="inlineStr"/>
@@ -1558,6 +2058,11 @@
       <c r="G86" s="3" t="inlineStr"/>
       <c r="H86" s="3" t="inlineStr"/>
       <c r="I86" s="3" t="inlineStr"/>
+      <c r="J86" s="3" t="inlineStr"/>
+      <c r="K86" s="3" t="inlineStr"/>
+      <c r="L86" s="3" t="inlineStr"/>
+      <c r="M86" s="3" t="inlineStr"/>
+      <c r="N86" s="3" t="inlineStr"/>
     </row>
     <row r="87" ht="18" customHeight="1">
       <c r="A87" s="3" t="inlineStr"/>
@@ -1569,6 +2074,11 @@
       <c r="G87" s="3" t="inlineStr"/>
       <c r="H87" s="3" t="inlineStr"/>
       <c r="I87" s="3" t="inlineStr"/>
+      <c r="J87" s="3" t="inlineStr"/>
+      <c r="K87" s="3" t="inlineStr"/>
+      <c r="L87" s="3" t="inlineStr"/>
+      <c r="M87" s="3" t="inlineStr"/>
+      <c r="N87" s="3" t="inlineStr"/>
     </row>
     <row r="88" ht="18" customHeight="1">
       <c r="A88" s="3" t="inlineStr"/>
@@ -1580,6 +2090,11 @@
       <c r="G88" s="3" t="inlineStr"/>
       <c r="H88" s="3" t="inlineStr"/>
       <c r="I88" s="3" t="inlineStr"/>
+      <c r="J88" s="3" t="inlineStr"/>
+      <c r="K88" s="3" t="inlineStr"/>
+      <c r="L88" s="3" t="inlineStr"/>
+      <c r="M88" s="3" t="inlineStr"/>
+      <c r="N88" s="3" t="inlineStr"/>
     </row>
     <row r="89" ht="18" customHeight="1">
       <c r="A89" s="3" t="inlineStr"/>
@@ -1591,6 +2106,11 @@
       <c r="G89" s="3" t="inlineStr"/>
       <c r="H89" s="3" t="inlineStr"/>
       <c r="I89" s="3" t="inlineStr"/>
+      <c r="J89" s="3" t="inlineStr"/>
+      <c r="K89" s="3" t="inlineStr"/>
+      <c r="L89" s="3" t="inlineStr"/>
+      <c r="M89" s="3" t="inlineStr"/>
+      <c r="N89" s="3" t="inlineStr"/>
     </row>
     <row r="90" ht="18" customHeight="1">
       <c r="A90" s="3" t="inlineStr"/>
@@ -1602,6 +2122,11 @@
       <c r="G90" s="3" t="inlineStr"/>
       <c r="H90" s="3" t="inlineStr"/>
       <c r="I90" s="3" t="inlineStr"/>
+      <c r="J90" s="3" t="inlineStr"/>
+      <c r="K90" s="3" t="inlineStr"/>
+      <c r="L90" s="3" t="inlineStr"/>
+      <c r="M90" s="3" t="inlineStr"/>
+      <c r="N90" s="3" t="inlineStr"/>
     </row>
     <row r="91" ht="18" customHeight="1">
       <c r="A91" s="3" t="inlineStr"/>
@@ -1613,6 +2138,11 @@
       <c r="G91" s="3" t="inlineStr"/>
       <c r="H91" s="3" t="inlineStr"/>
       <c r="I91" s="3" t="inlineStr"/>
+      <c r="J91" s="3" t="inlineStr"/>
+      <c r="K91" s="3" t="inlineStr"/>
+      <c r="L91" s="3" t="inlineStr"/>
+      <c r="M91" s="3" t="inlineStr"/>
+      <c r="N91" s="3" t="inlineStr"/>
     </row>
     <row r="92" ht="18" customHeight="1">
       <c r="A92" s="3" t="inlineStr"/>
@@ -1624,6 +2154,11 @@
       <c r="G92" s="3" t="inlineStr"/>
       <c r="H92" s="3" t="inlineStr"/>
       <c r="I92" s="3" t="inlineStr"/>
+      <c r="J92" s="3" t="inlineStr"/>
+      <c r="K92" s="3" t="inlineStr"/>
+      <c r="L92" s="3" t="inlineStr"/>
+      <c r="M92" s="3" t="inlineStr"/>
+      <c r="N92" s="3" t="inlineStr"/>
     </row>
     <row r="93" ht="18" customHeight="1">
       <c r="A93" s="3" t="inlineStr"/>
@@ -1635,6 +2170,11 @@
       <c r="G93" s="3" t="inlineStr"/>
       <c r="H93" s="3" t="inlineStr"/>
       <c r="I93" s="3" t="inlineStr"/>
+      <c r="J93" s="3" t="inlineStr"/>
+      <c r="K93" s="3" t="inlineStr"/>
+      <c r="L93" s="3" t="inlineStr"/>
+      <c r="M93" s="3" t="inlineStr"/>
+      <c r="N93" s="3" t="inlineStr"/>
     </row>
     <row r="94" ht="18" customHeight="1">
       <c r="A94" s="3" t="inlineStr"/>
@@ -1646,6 +2186,11 @@
       <c r="G94" s="3" t="inlineStr"/>
       <c r="H94" s="3" t="inlineStr"/>
       <c r="I94" s="3" t="inlineStr"/>
+      <c r="J94" s="3" t="inlineStr"/>
+      <c r="K94" s="3" t="inlineStr"/>
+      <c r="L94" s="3" t="inlineStr"/>
+      <c r="M94" s="3" t="inlineStr"/>
+      <c r="N94" s="3" t="inlineStr"/>
     </row>
     <row r="95" ht="18" customHeight="1">
       <c r="A95" s="3" t="inlineStr"/>
@@ -1657,6 +2202,11 @@
       <c r="G95" s="3" t="inlineStr"/>
       <c r="H95" s="3" t="inlineStr"/>
       <c r="I95" s="3" t="inlineStr"/>
+      <c r="J95" s="3" t="inlineStr"/>
+      <c r="K95" s="3" t="inlineStr"/>
+      <c r="L95" s="3" t="inlineStr"/>
+      <c r="M95" s="3" t="inlineStr"/>
+      <c r="N95" s="3" t="inlineStr"/>
     </row>
     <row r="96" ht="18" customHeight="1">
       <c r="A96" s="3" t="inlineStr"/>
@@ -1668,6 +2218,11 @@
       <c r="G96" s="3" t="inlineStr"/>
       <c r="H96" s="3" t="inlineStr"/>
       <c r="I96" s="3" t="inlineStr"/>
+      <c r="J96" s="3" t="inlineStr"/>
+      <c r="K96" s="3" t="inlineStr"/>
+      <c r="L96" s="3" t="inlineStr"/>
+      <c r="M96" s="3" t="inlineStr"/>
+      <c r="N96" s="3" t="inlineStr"/>
     </row>
     <row r="97" ht="18" customHeight="1">
       <c r="A97" s="3" t="inlineStr"/>
@@ -1679,6 +2234,11 @@
       <c r="G97" s="3" t="inlineStr"/>
       <c r="H97" s="3" t="inlineStr"/>
       <c r="I97" s="3" t="inlineStr"/>
+      <c r="J97" s="3" t="inlineStr"/>
+      <c r="K97" s="3" t="inlineStr"/>
+      <c r="L97" s="3" t="inlineStr"/>
+      <c r="M97" s="3" t="inlineStr"/>
+      <c r="N97" s="3" t="inlineStr"/>
     </row>
     <row r="98" ht="18" customHeight="1">
       <c r="A98" s="3" t="inlineStr"/>
@@ -1690,6 +2250,11 @@
       <c r="G98" s="3" t="inlineStr"/>
       <c r="H98" s="3" t="inlineStr"/>
       <c r="I98" s="3" t="inlineStr"/>
+      <c r="J98" s="3" t="inlineStr"/>
+      <c r="K98" s="3" t="inlineStr"/>
+      <c r="L98" s="3" t="inlineStr"/>
+      <c r="M98" s="3" t="inlineStr"/>
+      <c r="N98" s="3" t="inlineStr"/>
     </row>
     <row r="99" ht="18" customHeight="1">
       <c r="A99" s="3" t="inlineStr"/>
@@ -1701,6 +2266,11 @@
       <c r="G99" s="3" t="inlineStr"/>
       <c r="H99" s="3" t="inlineStr"/>
       <c r="I99" s="3" t="inlineStr"/>
+      <c r="J99" s="3" t="inlineStr"/>
+      <c r="K99" s="3" t="inlineStr"/>
+      <c r="L99" s="3" t="inlineStr"/>
+      <c r="M99" s="3" t="inlineStr"/>
+      <c r="N99" s="3" t="inlineStr"/>
     </row>
     <row r="100" ht="18" customHeight="1">
       <c r="A100" s="3" t="inlineStr"/>
@@ -1712,6 +2282,11 @@
       <c r="G100" s="3" t="inlineStr"/>
       <c r="H100" s="3" t="inlineStr"/>
       <c r="I100" s="3" t="inlineStr"/>
+      <c r="J100" s="3" t="inlineStr"/>
+      <c r="K100" s="3" t="inlineStr"/>
+      <c r="L100" s="3" t="inlineStr"/>
+      <c r="M100" s="3" t="inlineStr"/>
+      <c r="N100" s="3" t="inlineStr"/>
     </row>
     <row r="101" ht="18" customHeight="1">
       <c r="A101" s="3" t="inlineStr"/>
@@ -1723,6 +2298,11 @@
       <c r="G101" s="3" t="inlineStr"/>
       <c r="H101" s="3" t="inlineStr"/>
       <c r="I101" s="3" t="inlineStr"/>
+      <c r="J101" s="3" t="inlineStr"/>
+      <c r="K101" s="3" t="inlineStr"/>
+      <c r="L101" s="3" t="inlineStr"/>
+      <c r="M101" s="3" t="inlineStr"/>
+      <c r="N101" s="3" t="inlineStr"/>
     </row>
     <row r="102" ht="18" customHeight="1">
       <c r="A102" s="3" t="inlineStr"/>
@@ -1734,6 +2314,11 @@
       <c r="G102" s="3" t="inlineStr"/>
       <c r="H102" s="3" t="inlineStr"/>
       <c r="I102" s="3" t="inlineStr"/>
+      <c r="J102" s="3" t="inlineStr"/>
+      <c r="K102" s="3" t="inlineStr"/>
+      <c r="L102" s="3" t="inlineStr"/>
+      <c r="M102" s="3" t="inlineStr"/>
+      <c r="N102" s="3" t="inlineStr"/>
     </row>
     <row r="103" ht="18" customHeight="1">
       <c r="A103" s="3" t="inlineStr"/>
@@ -1745,6 +2330,11 @@
       <c r="G103" s="3" t="inlineStr"/>
       <c r="H103" s="3" t="inlineStr"/>
       <c r="I103" s="3" t="inlineStr"/>
+      <c r="J103" s="3" t="inlineStr"/>
+      <c r="K103" s="3" t="inlineStr"/>
+      <c r="L103" s="3" t="inlineStr"/>
+      <c r="M103" s="3" t="inlineStr"/>
+      <c r="N103" s="3" t="inlineStr"/>
     </row>
     <row r="104" ht="18" customHeight="1">
       <c r="A104" s="3" t="inlineStr"/>
@@ -1756,6 +2346,11 @@
       <c r="G104" s="3" t="inlineStr"/>
       <c r="H104" s="3" t="inlineStr"/>
       <c r="I104" s="3" t="inlineStr"/>
+      <c r="J104" s="3" t="inlineStr"/>
+      <c r="K104" s="3" t="inlineStr"/>
+      <c r="L104" s="3" t="inlineStr"/>
+      <c r="M104" s="3" t="inlineStr"/>
+      <c r="N104" s="3" t="inlineStr"/>
     </row>
     <row r="105" ht="18" customHeight="1">
       <c r="A105" s="3" t="inlineStr"/>
@@ -1767,6 +2362,11 @@
       <c r="G105" s="3" t="inlineStr"/>
       <c r="H105" s="3" t="inlineStr"/>
       <c r="I105" s="3" t="inlineStr"/>
+      <c r="J105" s="3" t="inlineStr"/>
+      <c r="K105" s="3" t="inlineStr"/>
+      <c r="L105" s="3" t="inlineStr"/>
+      <c r="M105" s="3" t="inlineStr"/>
+      <c r="N105" s="3" t="inlineStr"/>
     </row>
     <row r="106" ht="18" customHeight="1">
       <c r="A106" s="3" t="inlineStr"/>
@@ -1778,6 +2378,11 @@
       <c r="G106" s="3" t="inlineStr"/>
       <c r="H106" s="3" t="inlineStr"/>
       <c r="I106" s="3" t="inlineStr"/>
+      <c r="J106" s="3" t="inlineStr"/>
+      <c r="K106" s="3" t="inlineStr"/>
+      <c r="L106" s="3" t="inlineStr"/>
+      <c r="M106" s="3" t="inlineStr"/>
+      <c r="N106" s="3" t="inlineStr"/>
     </row>
     <row r="107" ht="18" customHeight="1">
       <c r="A107" s="3" t="inlineStr"/>
@@ -1789,6 +2394,11 @@
       <c r="G107" s="3" t="inlineStr"/>
       <c r="H107" s="3" t="inlineStr"/>
       <c r="I107" s="3" t="inlineStr"/>
+      <c r="J107" s="3" t="inlineStr"/>
+      <c r="K107" s="3" t="inlineStr"/>
+      <c r="L107" s="3" t="inlineStr"/>
+      <c r="M107" s="3" t="inlineStr"/>
+      <c r="N107" s="3" t="inlineStr"/>
     </row>
     <row r="108" ht="18" customHeight="1">
       <c r="A108" s="3" t="inlineStr"/>
@@ -1800,6 +2410,11 @@
       <c r="G108" s="3" t="inlineStr"/>
       <c r="H108" s="3" t="inlineStr"/>
       <c r="I108" s="3" t="inlineStr"/>
+      <c r="J108" s="3" t="inlineStr"/>
+      <c r="K108" s="3" t="inlineStr"/>
+      <c r="L108" s="3" t="inlineStr"/>
+      <c r="M108" s="3" t="inlineStr"/>
+      <c r="N108" s="3" t="inlineStr"/>
     </row>
     <row r="109" ht="18" customHeight="1">
       <c r="A109" s="3" t="inlineStr"/>
@@ -1811,6 +2426,11 @@
       <c r="G109" s="3" t="inlineStr"/>
       <c r="H109" s="3" t="inlineStr"/>
       <c r="I109" s="3" t="inlineStr"/>
+      <c r="J109" s="3" t="inlineStr"/>
+      <c r="K109" s="3" t="inlineStr"/>
+      <c r="L109" s="3" t="inlineStr"/>
+      <c r="M109" s="3" t="inlineStr"/>
+      <c r="N109" s="3" t="inlineStr"/>
     </row>
     <row r="110" ht="18" customHeight="1">
       <c r="A110" s="3" t="inlineStr"/>
@@ -1822,6 +2442,11 @@
       <c r="G110" s="3" t="inlineStr"/>
       <c r="H110" s="3" t="inlineStr"/>
       <c r="I110" s="3" t="inlineStr"/>
+      <c r="J110" s="3" t="inlineStr"/>
+      <c r="K110" s="3" t="inlineStr"/>
+      <c r="L110" s="3" t="inlineStr"/>
+      <c r="M110" s="3" t="inlineStr"/>
+      <c r="N110" s="3" t="inlineStr"/>
     </row>
     <row r="111" ht="18" customHeight="1">
       <c r="A111" s="3" t="inlineStr"/>
@@ -1833,6 +2458,11 @@
       <c r="G111" s="3" t="inlineStr"/>
       <c r="H111" s="3" t="inlineStr"/>
       <c r="I111" s="3" t="inlineStr"/>
+      <c r="J111" s="3" t="inlineStr"/>
+      <c r="K111" s="3" t="inlineStr"/>
+      <c r="L111" s="3" t="inlineStr"/>
+      <c r="M111" s="3" t="inlineStr"/>
+      <c r="N111" s="3" t="inlineStr"/>
     </row>
     <row r="112" ht="18" customHeight="1">
       <c r="A112" s="3" t="inlineStr"/>
@@ -1844,6 +2474,11 @@
       <c r="G112" s="3" t="inlineStr"/>
       <c r="H112" s="3" t="inlineStr"/>
       <c r="I112" s="3" t="inlineStr"/>
+      <c r="J112" s="3" t="inlineStr"/>
+      <c r="K112" s="3" t="inlineStr"/>
+      <c r="L112" s="3" t="inlineStr"/>
+      <c r="M112" s="3" t="inlineStr"/>
+      <c r="N112" s="3" t="inlineStr"/>
     </row>
     <row r="113" ht="18" customHeight="1">
       <c r="A113" s="3" t="inlineStr"/>
@@ -1855,6 +2490,11 @@
       <c r="G113" s="3" t="inlineStr"/>
       <c r="H113" s="3" t="inlineStr"/>
       <c r="I113" s="3" t="inlineStr"/>
+      <c r="J113" s="3" t="inlineStr"/>
+      <c r="K113" s="3" t="inlineStr"/>
+      <c r="L113" s="3" t="inlineStr"/>
+      <c r="M113" s="3" t="inlineStr"/>
+      <c r="N113" s="3" t="inlineStr"/>
     </row>
     <row r="114" ht="18" customHeight="1">
       <c r="A114" s="3" t="inlineStr"/>
@@ -1866,6 +2506,11 @@
       <c r="G114" s="3" t="inlineStr"/>
       <c r="H114" s="3" t="inlineStr"/>
       <c r="I114" s="3" t="inlineStr"/>
+      <c r="J114" s="3" t="inlineStr"/>
+      <c r="K114" s="3" t="inlineStr"/>
+      <c r="L114" s="3" t="inlineStr"/>
+      <c r="M114" s="3" t="inlineStr"/>
+      <c r="N114" s="3" t="inlineStr"/>
     </row>
     <row r="115" ht="18" customHeight="1">
       <c r="A115" s="3" t="inlineStr"/>
@@ -1877,6 +2522,11 @@
       <c r="G115" s="3" t="inlineStr"/>
       <c r="H115" s="3" t="inlineStr"/>
       <c r="I115" s="3" t="inlineStr"/>
+      <c r="J115" s="3" t="inlineStr"/>
+      <c r="K115" s="3" t="inlineStr"/>
+      <c r="L115" s="3" t="inlineStr"/>
+      <c r="M115" s="3" t="inlineStr"/>
+      <c r="N115" s="3" t="inlineStr"/>
     </row>
     <row r="116" ht="18" customHeight="1">
       <c r="A116" s="3" t="inlineStr"/>
@@ -1888,6 +2538,11 @@
       <c r="G116" s="3" t="inlineStr"/>
       <c r="H116" s="3" t="inlineStr"/>
       <c r="I116" s="3" t="inlineStr"/>
+      <c r="J116" s="3" t="inlineStr"/>
+      <c r="K116" s="3" t="inlineStr"/>
+      <c r="L116" s="3" t="inlineStr"/>
+      <c r="M116" s="3" t="inlineStr"/>
+      <c r="N116" s="3" t="inlineStr"/>
     </row>
     <row r="117" ht="18" customHeight="1">
       <c r="A117" s="3" t="inlineStr"/>
@@ -1899,6 +2554,11 @@
       <c r="G117" s="3" t="inlineStr"/>
       <c r="H117" s="3" t="inlineStr"/>
       <c r="I117" s="3" t="inlineStr"/>
+      <c r="J117" s="3" t="inlineStr"/>
+      <c r="K117" s="3" t="inlineStr"/>
+      <c r="L117" s="3" t="inlineStr"/>
+      <c r="M117" s="3" t="inlineStr"/>
+      <c r="N117" s="3" t="inlineStr"/>
     </row>
     <row r="118" ht="18" customHeight="1">
       <c r="A118" s="3" t="inlineStr"/>
@@ -1910,6 +2570,11 @@
       <c r="G118" s="3" t="inlineStr"/>
       <c r="H118" s="3" t="inlineStr"/>
       <c r="I118" s="3" t="inlineStr"/>
+      <c r="J118" s="3" t="inlineStr"/>
+      <c r="K118" s="3" t="inlineStr"/>
+      <c r="L118" s="3" t="inlineStr"/>
+      <c r="M118" s="3" t="inlineStr"/>
+      <c r="N118" s="3" t="inlineStr"/>
     </row>
     <row r="119" ht="18" customHeight="1">
       <c r="A119" s="3" t="inlineStr"/>
@@ -1921,6 +2586,11 @@
       <c r="G119" s="3" t="inlineStr"/>
       <c r="H119" s="3" t="inlineStr"/>
       <c r="I119" s="3" t="inlineStr"/>
+      <c r="J119" s="3" t="inlineStr"/>
+      <c r="K119" s="3" t="inlineStr"/>
+      <c r="L119" s="3" t="inlineStr"/>
+      <c r="M119" s="3" t="inlineStr"/>
+      <c r="N119" s="3" t="inlineStr"/>
     </row>
     <row r="120" ht="18" customHeight="1">
       <c r="A120" s="3" t="inlineStr"/>
@@ -1932,6 +2602,11 @@
       <c r="G120" s="3" t="inlineStr"/>
       <c r="H120" s="3" t="inlineStr"/>
       <c r="I120" s="3" t="inlineStr"/>
+      <c r="J120" s="3" t="inlineStr"/>
+      <c r="K120" s="3" t="inlineStr"/>
+      <c r="L120" s="3" t="inlineStr"/>
+      <c r="M120" s="3" t="inlineStr"/>
+      <c r="N120" s="3" t="inlineStr"/>
     </row>
     <row r="121" ht="18" customHeight="1">
       <c r="A121" s="3" t="inlineStr"/>
@@ -1943,6 +2618,11 @@
       <c r="G121" s="3" t="inlineStr"/>
       <c r="H121" s="3" t="inlineStr"/>
       <c r="I121" s="3" t="inlineStr"/>
+      <c r="J121" s="3" t="inlineStr"/>
+      <c r="K121" s="3" t="inlineStr"/>
+      <c r="L121" s="3" t="inlineStr"/>
+      <c r="M121" s="3" t="inlineStr"/>
+      <c r="N121" s="3" t="inlineStr"/>
     </row>
     <row r="122" ht="18" customHeight="1">
       <c r="A122" s="3" t="inlineStr"/>
@@ -1954,6 +2634,11 @@
       <c r="G122" s="3" t="inlineStr"/>
       <c r="H122" s="3" t="inlineStr"/>
       <c r="I122" s="3" t="inlineStr"/>
+      <c r="J122" s="3" t="inlineStr"/>
+      <c r="K122" s="3" t="inlineStr"/>
+      <c r="L122" s="3" t="inlineStr"/>
+      <c r="M122" s="3" t="inlineStr"/>
+      <c r="N122" s="3" t="inlineStr"/>
     </row>
     <row r="123" ht="18" customHeight="1">
       <c r="A123" s="3" t="inlineStr"/>
@@ -1965,6 +2650,11 @@
       <c r="G123" s="3" t="inlineStr"/>
       <c r="H123" s="3" t="inlineStr"/>
       <c r="I123" s="3" t="inlineStr"/>
+      <c r="J123" s="3" t="inlineStr"/>
+      <c r="K123" s="3" t="inlineStr"/>
+      <c r="L123" s="3" t="inlineStr"/>
+      <c r="M123" s="3" t="inlineStr"/>
+      <c r="N123" s="3" t="inlineStr"/>
     </row>
     <row r="124" ht="18" customHeight="1">
       <c r="A124" s="3" t="inlineStr"/>
@@ -1976,6 +2666,11 @@
       <c r="G124" s="3" t="inlineStr"/>
       <c r="H124" s="3" t="inlineStr"/>
       <c r="I124" s="3" t="inlineStr"/>
+      <c r="J124" s="3" t="inlineStr"/>
+      <c r="K124" s="3" t="inlineStr"/>
+      <c r="L124" s="3" t="inlineStr"/>
+      <c r="M124" s="3" t="inlineStr"/>
+      <c r="N124" s="3" t="inlineStr"/>
     </row>
     <row r="125" ht="18" customHeight="1">
       <c r="A125" s="3" t="inlineStr"/>
@@ -1987,6 +2682,11 @@
       <c r="G125" s="3" t="inlineStr"/>
       <c r="H125" s="3" t="inlineStr"/>
       <c r="I125" s="3" t="inlineStr"/>
+      <c r="J125" s="3" t="inlineStr"/>
+      <c r="K125" s="3" t="inlineStr"/>
+      <c r="L125" s="3" t="inlineStr"/>
+      <c r="M125" s="3" t="inlineStr"/>
+      <c r="N125" s="3" t="inlineStr"/>
     </row>
     <row r="126" ht="18" customHeight="1">
       <c r="A126" s="3" t="inlineStr"/>
@@ -1998,6 +2698,11 @@
       <c r="G126" s="3" t="inlineStr"/>
       <c r="H126" s="3" t="inlineStr"/>
       <c r="I126" s="3" t="inlineStr"/>
+      <c r="J126" s="3" t="inlineStr"/>
+      <c r="K126" s="3" t="inlineStr"/>
+      <c r="L126" s="3" t="inlineStr"/>
+      <c r="M126" s="3" t="inlineStr"/>
+      <c r="N126" s="3" t="inlineStr"/>
     </row>
     <row r="127" ht="18" customHeight="1">
       <c r="A127" s="3" t="inlineStr"/>
@@ -2009,6 +2714,11 @@
       <c r="G127" s="3" t="inlineStr"/>
       <c r="H127" s="3" t="inlineStr"/>
       <c r="I127" s="3" t="inlineStr"/>
+      <c r="J127" s="3" t="inlineStr"/>
+      <c r="K127" s="3" t="inlineStr"/>
+      <c r="L127" s="3" t="inlineStr"/>
+      <c r="M127" s="3" t="inlineStr"/>
+      <c r="N127" s="3" t="inlineStr"/>
     </row>
     <row r="128" ht="18" customHeight="1">
       <c r="A128" s="3" t="inlineStr"/>
@@ -2020,6 +2730,11 @@
       <c r="G128" s="3" t="inlineStr"/>
       <c r="H128" s="3" t="inlineStr"/>
       <c r="I128" s="3" t="inlineStr"/>
+      <c r="J128" s="3" t="inlineStr"/>
+      <c r="K128" s="3" t="inlineStr"/>
+      <c r="L128" s="3" t="inlineStr"/>
+      <c r="M128" s="3" t="inlineStr"/>
+      <c r="N128" s="3" t="inlineStr"/>
     </row>
     <row r="129" ht="18" customHeight="1">
       <c r="A129" s="3" t="inlineStr"/>
@@ -2031,6 +2746,11 @@
       <c r="G129" s="3" t="inlineStr"/>
       <c r="H129" s="3" t="inlineStr"/>
       <c r="I129" s="3" t="inlineStr"/>
+      <c r="J129" s="3" t="inlineStr"/>
+      <c r="K129" s="3" t="inlineStr"/>
+      <c r="L129" s="3" t="inlineStr"/>
+      <c r="M129" s="3" t="inlineStr"/>
+      <c r="N129" s="3" t="inlineStr"/>
     </row>
     <row r="130" ht="18" customHeight="1">
       <c r="A130" s="3" t="inlineStr"/>
@@ -2042,6 +2762,11 @@
       <c r="G130" s="3" t="inlineStr"/>
       <c r="H130" s="3" t="inlineStr"/>
       <c r="I130" s="3" t="inlineStr"/>
+      <c r="J130" s="3" t="inlineStr"/>
+      <c r="K130" s="3" t="inlineStr"/>
+      <c r="L130" s="3" t="inlineStr"/>
+      <c r="M130" s="3" t="inlineStr"/>
+      <c r="N130" s="3" t="inlineStr"/>
     </row>
     <row r="131" ht="18" customHeight="1">
       <c r="A131" s="3" t="inlineStr"/>
@@ -2053,6 +2778,11 @@
       <c r="G131" s="3" t="inlineStr"/>
       <c r="H131" s="3" t="inlineStr"/>
       <c r="I131" s="3" t="inlineStr"/>
+      <c r="J131" s="3" t="inlineStr"/>
+      <c r="K131" s="3" t="inlineStr"/>
+      <c r="L131" s="3" t="inlineStr"/>
+      <c r="M131" s="3" t="inlineStr"/>
+      <c r="N131" s="3" t="inlineStr"/>
     </row>
     <row r="132" ht="18" customHeight="1">
       <c r="A132" s="3" t="inlineStr"/>
@@ -2064,6 +2794,11 @@
       <c r="G132" s="3" t="inlineStr"/>
       <c r="H132" s="3" t="inlineStr"/>
       <c r="I132" s="3" t="inlineStr"/>
+      <c r="J132" s="3" t="inlineStr"/>
+      <c r="K132" s="3" t="inlineStr"/>
+      <c r="L132" s="3" t="inlineStr"/>
+      <c r="M132" s="3" t="inlineStr"/>
+      <c r="N132" s="3" t="inlineStr"/>
     </row>
     <row r="133" ht="18" customHeight="1">
       <c r="A133" s="3" t="inlineStr"/>
@@ -2075,6 +2810,11 @@
       <c r="G133" s="3" t="inlineStr"/>
       <c r="H133" s="3" t="inlineStr"/>
       <c r="I133" s="3" t="inlineStr"/>
+      <c r="J133" s="3" t="inlineStr"/>
+      <c r="K133" s="3" t="inlineStr"/>
+      <c r="L133" s="3" t="inlineStr"/>
+      <c r="M133" s="3" t="inlineStr"/>
+      <c r="N133" s="3" t="inlineStr"/>
     </row>
     <row r="134" ht="18" customHeight="1">
       <c r="A134" s="3" t="inlineStr"/>
@@ -2086,6 +2826,11 @@
       <c r="G134" s="3" t="inlineStr"/>
       <c r="H134" s="3" t="inlineStr"/>
       <c r="I134" s="3" t="inlineStr"/>
+      <c r="J134" s="3" t="inlineStr"/>
+      <c r="K134" s="3" t="inlineStr"/>
+      <c r="L134" s="3" t="inlineStr"/>
+      <c r="M134" s="3" t="inlineStr"/>
+      <c r="N134" s="3" t="inlineStr"/>
     </row>
     <row r="135" ht="18" customHeight="1">
       <c r="A135" s="3" t="inlineStr"/>
@@ -2097,6 +2842,11 @@
       <c r="G135" s="3" t="inlineStr"/>
       <c r="H135" s="3" t="inlineStr"/>
       <c r="I135" s="3" t="inlineStr"/>
+      <c r="J135" s="3" t="inlineStr"/>
+      <c r="K135" s="3" t="inlineStr"/>
+      <c r="L135" s="3" t="inlineStr"/>
+      <c r="M135" s="3" t="inlineStr"/>
+      <c r="N135" s="3" t="inlineStr"/>
     </row>
     <row r="136" ht="18" customHeight="1">
       <c r="A136" s="3" t="inlineStr"/>
@@ -2108,6 +2858,11 @@
       <c r="G136" s="3" t="inlineStr"/>
       <c r="H136" s="3" t="inlineStr"/>
       <c r="I136" s="3" t="inlineStr"/>
+      <c r="J136" s="3" t="inlineStr"/>
+      <c r="K136" s="3" t="inlineStr"/>
+      <c r="L136" s="3" t="inlineStr"/>
+      <c r="M136" s="3" t="inlineStr"/>
+      <c r="N136" s="3" t="inlineStr"/>
     </row>
     <row r="137" ht="18" customHeight="1">
       <c r="A137" s="3" t="inlineStr"/>
@@ -2119,6 +2874,11 @@
       <c r="G137" s="3" t="inlineStr"/>
       <c r="H137" s="3" t="inlineStr"/>
       <c r="I137" s="3" t="inlineStr"/>
+      <c r="J137" s="3" t="inlineStr"/>
+      <c r="K137" s="3" t="inlineStr"/>
+      <c r="L137" s="3" t="inlineStr"/>
+      <c r="M137" s="3" t="inlineStr"/>
+      <c r="N137" s="3" t="inlineStr"/>
     </row>
     <row r="138" ht="18" customHeight="1">
       <c r="A138" s="3" t="inlineStr"/>
@@ -2130,6 +2890,11 @@
       <c r="G138" s="3" t="inlineStr"/>
       <c r="H138" s="3" t="inlineStr"/>
       <c r="I138" s="3" t="inlineStr"/>
+      <c r="J138" s="3" t="inlineStr"/>
+      <c r="K138" s="3" t="inlineStr"/>
+      <c r="L138" s="3" t="inlineStr"/>
+      <c r="M138" s="3" t="inlineStr"/>
+      <c r="N138" s="3" t="inlineStr"/>
     </row>
     <row r="139" ht="18" customHeight="1">
       <c r="A139" s="3" t="inlineStr"/>
@@ -2141,6 +2906,11 @@
       <c r="G139" s="3" t="inlineStr"/>
       <c r="H139" s="3" t="inlineStr"/>
       <c r="I139" s="3" t="inlineStr"/>
+      <c r="J139" s="3" t="inlineStr"/>
+      <c r="K139" s="3" t="inlineStr"/>
+      <c r="L139" s="3" t="inlineStr"/>
+      <c r="M139" s="3" t="inlineStr"/>
+      <c r="N139" s="3" t="inlineStr"/>
     </row>
     <row r="140" ht="18" customHeight="1">
       <c r="A140" s="3" t="inlineStr"/>
@@ -2152,6 +2922,11 @@
       <c r="G140" s="3" t="inlineStr"/>
       <c r="H140" s="3" t="inlineStr"/>
       <c r="I140" s="3" t="inlineStr"/>
+      <c r="J140" s="3" t="inlineStr"/>
+      <c r="K140" s="3" t="inlineStr"/>
+      <c r="L140" s="3" t="inlineStr"/>
+      <c r="M140" s="3" t="inlineStr"/>
+      <c r="N140" s="3" t="inlineStr"/>
     </row>
     <row r="141" ht="18" customHeight="1">
       <c r="A141" s="3" t="inlineStr"/>
@@ -2163,6 +2938,11 @@
       <c r="G141" s="3" t="inlineStr"/>
       <c r="H141" s="3" t="inlineStr"/>
       <c r="I141" s="3" t="inlineStr"/>
+      <c r="J141" s="3" t="inlineStr"/>
+      <c r="K141" s="3" t="inlineStr"/>
+      <c r="L141" s="3" t="inlineStr"/>
+      <c r="M141" s="3" t="inlineStr"/>
+      <c r="N141" s="3" t="inlineStr"/>
     </row>
     <row r="142" ht="18" customHeight="1">
       <c r="A142" s="3" t="inlineStr"/>
@@ -2174,6 +2954,11 @@
       <c r="G142" s="3" t="inlineStr"/>
       <c r="H142" s="3" t="inlineStr"/>
       <c r="I142" s="3" t="inlineStr"/>
+      <c r="J142" s="3" t="inlineStr"/>
+      <c r="K142" s="3" t="inlineStr"/>
+      <c r="L142" s="3" t="inlineStr"/>
+      <c r="M142" s="3" t="inlineStr"/>
+      <c r="N142" s="3" t="inlineStr"/>
     </row>
     <row r="143" ht="18" customHeight="1">
       <c r="A143" s="3" t="inlineStr"/>
@@ -2185,6 +2970,11 @@
       <c r="G143" s="3" t="inlineStr"/>
       <c r="H143" s="3" t="inlineStr"/>
       <c r="I143" s="3" t="inlineStr"/>
+      <c r="J143" s="3" t="inlineStr"/>
+      <c r="K143" s="3" t="inlineStr"/>
+      <c r="L143" s="3" t="inlineStr"/>
+      <c r="M143" s="3" t="inlineStr"/>
+      <c r="N143" s="3" t="inlineStr"/>
     </row>
     <row r="144" ht="18" customHeight="1">
       <c r="A144" s="3" t="inlineStr"/>
@@ -2196,6 +2986,11 @@
       <c r="G144" s="3" t="inlineStr"/>
       <c r="H144" s="3" t="inlineStr"/>
       <c r="I144" s="3" t="inlineStr"/>
+      <c r="J144" s="3" t="inlineStr"/>
+      <c r="K144" s="3" t="inlineStr"/>
+      <c r="L144" s="3" t="inlineStr"/>
+      <c r="M144" s="3" t="inlineStr"/>
+      <c r="N144" s="3" t="inlineStr"/>
     </row>
     <row r="145" ht="18" customHeight="1">
       <c r="A145" s="3" t="inlineStr"/>
@@ -2207,6 +3002,11 @@
       <c r="G145" s="3" t="inlineStr"/>
       <c r="H145" s="3" t="inlineStr"/>
       <c r="I145" s="3" t="inlineStr"/>
+      <c r="J145" s="3" t="inlineStr"/>
+      <c r="K145" s="3" t="inlineStr"/>
+      <c r="L145" s="3" t="inlineStr"/>
+      <c r="M145" s="3" t="inlineStr"/>
+      <c r="N145" s="3" t="inlineStr"/>
     </row>
     <row r="146" ht="18" customHeight="1">
       <c r="A146" s="3" t="inlineStr"/>
@@ -2218,6 +3018,11 @@
       <c r="G146" s="3" t="inlineStr"/>
       <c r="H146" s="3" t="inlineStr"/>
       <c r="I146" s="3" t="inlineStr"/>
+      <c r="J146" s="3" t="inlineStr"/>
+      <c r="K146" s="3" t="inlineStr"/>
+      <c r="L146" s="3" t="inlineStr"/>
+      <c r="M146" s="3" t="inlineStr"/>
+      <c r="N146" s="3" t="inlineStr"/>
     </row>
     <row r="147" ht="18" customHeight="1">
       <c r="A147" s="3" t="inlineStr"/>
@@ -2229,6 +3034,11 @@
       <c r="G147" s="3" t="inlineStr"/>
       <c r="H147" s="3" t="inlineStr"/>
       <c r="I147" s="3" t="inlineStr"/>
+      <c r="J147" s="3" t="inlineStr"/>
+      <c r="K147" s="3" t="inlineStr"/>
+      <c r="L147" s="3" t="inlineStr"/>
+      <c r="M147" s="3" t="inlineStr"/>
+      <c r="N147" s="3" t="inlineStr"/>
     </row>
     <row r="148" ht="18" customHeight="1">
       <c r="A148" s="3" t="inlineStr"/>
@@ -2240,6 +3050,11 @@
       <c r="G148" s="3" t="inlineStr"/>
       <c r="H148" s="3" t="inlineStr"/>
       <c r="I148" s="3" t="inlineStr"/>
+      <c r="J148" s="3" t="inlineStr"/>
+      <c r="K148" s="3" t="inlineStr"/>
+      <c r="L148" s="3" t="inlineStr"/>
+      <c r="M148" s="3" t="inlineStr"/>
+      <c r="N148" s="3" t="inlineStr"/>
     </row>
     <row r="149" ht="18" customHeight="1">
       <c r="A149" s="3" t="inlineStr"/>
@@ -2251,6 +3066,11 @@
       <c r="G149" s="3" t="inlineStr"/>
       <c r="H149" s="3" t="inlineStr"/>
       <c r="I149" s="3" t="inlineStr"/>
+      <c r="J149" s="3" t="inlineStr"/>
+      <c r="K149" s="3" t="inlineStr"/>
+      <c r="L149" s="3" t="inlineStr"/>
+      <c r="M149" s="3" t="inlineStr"/>
+      <c r="N149" s="3" t="inlineStr"/>
     </row>
     <row r="150" ht="18" customHeight="1">
       <c r="A150" s="3" t="inlineStr"/>
@@ -2262,6 +3082,11 @@
       <c r="G150" s="3" t="inlineStr"/>
       <c r="H150" s="3" t="inlineStr"/>
       <c r="I150" s="3" t="inlineStr"/>
+      <c r="J150" s="3" t="inlineStr"/>
+      <c r="K150" s="3" t="inlineStr"/>
+      <c r="L150" s="3" t="inlineStr"/>
+      <c r="M150" s="3" t="inlineStr"/>
+      <c r="N150" s="3" t="inlineStr"/>
     </row>
     <row r="151" ht="18" customHeight="1">
       <c r="A151" s="3" t="inlineStr"/>
@@ -2273,6 +3098,11 @@
       <c r="G151" s="3" t="inlineStr"/>
       <c r="H151" s="3" t="inlineStr"/>
       <c r="I151" s="3" t="inlineStr"/>
+      <c r="J151" s="3" t="inlineStr"/>
+      <c r="K151" s="3" t="inlineStr"/>
+      <c r="L151" s="3" t="inlineStr"/>
+      <c r="M151" s="3" t="inlineStr"/>
+      <c r="N151" s="3" t="inlineStr"/>
     </row>
     <row r="152" ht="18" customHeight="1">
       <c r="A152" s="3" t="inlineStr"/>
@@ -2284,6 +3114,11 @@
       <c r="G152" s="3" t="inlineStr"/>
       <c r="H152" s="3" t="inlineStr"/>
       <c r="I152" s="3" t="inlineStr"/>
+      <c r="J152" s="3" t="inlineStr"/>
+      <c r="K152" s="3" t="inlineStr"/>
+      <c r="L152" s="3" t="inlineStr"/>
+      <c r="M152" s="3" t="inlineStr"/>
+      <c r="N152" s="3" t="inlineStr"/>
     </row>
     <row r="153" ht="18" customHeight="1">
       <c r="A153" s="3" t="inlineStr"/>
@@ -2295,6 +3130,11 @@
       <c r="G153" s="3" t="inlineStr"/>
       <c r="H153" s="3" t="inlineStr"/>
       <c r="I153" s="3" t="inlineStr"/>
+      <c r="J153" s="3" t="inlineStr"/>
+      <c r="K153" s="3" t="inlineStr"/>
+      <c r="L153" s="3" t="inlineStr"/>
+      <c r="M153" s="3" t="inlineStr"/>
+      <c r="N153" s="3" t="inlineStr"/>
     </row>
     <row r="154" ht="18" customHeight="1">
       <c r="A154" s="3" t="inlineStr"/>
@@ -2306,6 +3146,11 @@
       <c r="G154" s="3" t="inlineStr"/>
       <c r="H154" s="3" t="inlineStr"/>
       <c r="I154" s="3" t="inlineStr"/>
+      <c r="J154" s="3" t="inlineStr"/>
+      <c r="K154" s="3" t="inlineStr"/>
+      <c r="L154" s="3" t="inlineStr"/>
+      <c r="M154" s="3" t="inlineStr"/>
+      <c r="N154" s="3" t="inlineStr"/>
     </row>
     <row r="155" ht="18" customHeight="1">
       <c r="A155" s="3" t="inlineStr"/>
@@ -2317,6 +3162,11 @@
       <c r="G155" s="3" t="inlineStr"/>
       <c r="H155" s="3" t="inlineStr"/>
       <c r="I155" s="3" t="inlineStr"/>
+      <c r="J155" s="3" t="inlineStr"/>
+      <c r="K155" s="3" t="inlineStr"/>
+      <c r="L155" s="3" t="inlineStr"/>
+      <c r="M155" s="3" t="inlineStr"/>
+      <c r="N155" s="3" t="inlineStr"/>
     </row>
     <row r="156" ht="18" customHeight="1">
       <c r="A156" s="3" t="inlineStr"/>
@@ -2328,6 +3178,11 @@
       <c r="G156" s="3" t="inlineStr"/>
       <c r="H156" s="3" t="inlineStr"/>
       <c r="I156" s="3" t="inlineStr"/>
+      <c r="J156" s="3" t="inlineStr"/>
+      <c r="K156" s="3" t="inlineStr"/>
+      <c r="L156" s="3" t="inlineStr"/>
+      <c r="M156" s="3" t="inlineStr"/>
+      <c r="N156" s="3" t="inlineStr"/>
     </row>
     <row r="157" ht="18" customHeight="1">
       <c r="A157" s="3" t="inlineStr"/>
@@ -2339,6 +3194,11 @@
       <c r="G157" s="3" t="inlineStr"/>
       <c r="H157" s="3" t="inlineStr"/>
       <c r="I157" s="3" t="inlineStr"/>
+      <c r="J157" s="3" t="inlineStr"/>
+      <c r="K157" s="3" t="inlineStr"/>
+      <c r="L157" s="3" t="inlineStr"/>
+      <c r="M157" s="3" t="inlineStr"/>
+      <c r="N157" s="3" t="inlineStr"/>
     </row>
     <row r="158" ht="18" customHeight="1">
       <c r="A158" s="3" t="inlineStr"/>
@@ -2350,6 +3210,11 @@
       <c r="G158" s="3" t="inlineStr"/>
       <c r="H158" s="3" t="inlineStr"/>
       <c r="I158" s="3" t="inlineStr"/>
+      <c r="J158" s="3" t="inlineStr"/>
+      <c r="K158" s="3" t="inlineStr"/>
+      <c r="L158" s="3" t="inlineStr"/>
+      <c r="M158" s="3" t="inlineStr"/>
+      <c r="N158" s="3" t="inlineStr"/>
     </row>
     <row r="159" ht="18" customHeight="1">
       <c r="A159" s="3" t="inlineStr"/>
@@ -2361,6 +3226,11 @@
       <c r="G159" s="3" t="inlineStr"/>
       <c r="H159" s="3" t="inlineStr"/>
       <c r="I159" s="3" t="inlineStr"/>
+      <c r="J159" s="3" t="inlineStr"/>
+      <c r="K159" s="3" t="inlineStr"/>
+      <c r="L159" s="3" t="inlineStr"/>
+      <c r="M159" s="3" t="inlineStr"/>
+      <c r="N159" s="3" t="inlineStr"/>
     </row>
     <row r="160" ht="18" customHeight="1">
       <c r="A160" s="3" t="inlineStr"/>
@@ -2372,6 +3242,11 @@
       <c r="G160" s="3" t="inlineStr"/>
       <c r="H160" s="3" t="inlineStr"/>
       <c r="I160" s="3" t="inlineStr"/>
+      <c r="J160" s="3" t="inlineStr"/>
+      <c r="K160" s="3" t="inlineStr"/>
+      <c r="L160" s="3" t="inlineStr"/>
+      <c r="M160" s="3" t="inlineStr"/>
+      <c r="N160" s="3" t="inlineStr"/>
     </row>
     <row r="161" ht="18" customHeight="1">
       <c r="A161" s="3" t="inlineStr"/>
@@ -2383,6 +3258,11 @@
       <c r="G161" s="3" t="inlineStr"/>
       <c r="H161" s="3" t="inlineStr"/>
       <c r="I161" s="3" t="inlineStr"/>
+      <c r="J161" s="3" t="inlineStr"/>
+      <c r="K161" s="3" t="inlineStr"/>
+      <c r="L161" s="3" t="inlineStr"/>
+      <c r="M161" s="3" t="inlineStr"/>
+      <c r="N161" s="3" t="inlineStr"/>
     </row>
     <row r="162" ht="18" customHeight="1">
       <c r="A162" s="3" t="inlineStr"/>
@@ -2394,6 +3274,11 @@
       <c r="G162" s="3" t="inlineStr"/>
       <c r="H162" s="3" t="inlineStr"/>
       <c r="I162" s="3" t="inlineStr"/>
+      <c r="J162" s="3" t="inlineStr"/>
+      <c r="K162" s="3" t="inlineStr"/>
+      <c r="L162" s="3" t="inlineStr"/>
+      <c r="M162" s="3" t="inlineStr"/>
+      <c r="N162" s="3" t="inlineStr"/>
     </row>
     <row r="163" ht="18" customHeight="1">
       <c r="A163" s="3" t="inlineStr"/>
@@ -2405,6 +3290,11 @@
       <c r="G163" s="3" t="inlineStr"/>
       <c r="H163" s="3" t="inlineStr"/>
       <c r="I163" s="3" t="inlineStr"/>
+      <c r="J163" s="3" t="inlineStr"/>
+      <c r="K163" s="3" t="inlineStr"/>
+      <c r="L163" s="3" t="inlineStr"/>
+      <c r="M163" s="3" t="inlineStr"/>
+      <c r="N163" s="3" t="inlineStr"/>
     </row>
     <row r="164" ht="18" customHeight="1">
       <c r="A164" s="3" t="inlineStr"/>
@@ -2416,6 +3306,11 @@
       <c r="G164" s="3" t="inlineStr"/>
       <c r="H164" s="3" t="inlineStr"/>
       <c r="I164" s="3" t="inlineStr"/>
+      <c r="J164" s="3" t="inlineStr"/>
+      <c r="K164" s="3" t="inlineStr"/>
+      <c r="L164" s="3" t="inlineStr"/>
+      <c r="M164" s="3" t="inlineStr"/>
+      <c r="N164" s="3" t="inlineStr"/>
     </row>
     <row r="165" ht="18" customHeight="1">
       <c r="A165" s="3" t="inlineStr"/>
@@ -2427,6 +3322,11 @@
       <c r="G165" s="3" t="inlineStr"/>
       <c r="H165" s="3" t="inlineStr"/>
       <c r="I165" s="3" t="inlineStr"/>
+      <c r="J165" s="3" t="inlineStr"/>
+      <c r="K165" s="3" t="inlineStr"/>
+      <c r="L165" s="3" t="inlineStr"/>
+      <c r="M165" s="3" t="inlineStr"/>
+      <c r="N165" s="3" t="inlineStr"/>
     </row>
     <row r="166" ht="18" customHeight="1">
       <c r="A166" s="3" t="inlineStr"/>
@@ -2438,6 +3338,11 @@
       <c r="G166" s="3" t="inlineStr"/>
       <c r="H166" s="3" t="inlineStr"/>
       <c r="I166" s="3" t="inlineStr"/>
+      <c r="J166" s="3" t="inlineStr"/>
+      <c r="K166" s="3" t="inlineStr"/>
+      <c r="L166" s="3" t="inlineStr"/>
+      <c r="M166" s="3" t="inlineStr"/>
+      <c r="N166" s="3" t="inlineStr"/>
     </row>
     <row r="167" ht="18" customHeight="1">
       <c r="A167" s="3" t="inlineStr"/>
@@ -2449,6 +3354,11 @@
       <c r="G167" s="3" t="inlineStr"/>
       <c r="H167" s="3" t="inlineStr"/>
       <c r="I167" s="3" t="inlineStr"/>
+      <c r="J167" s="3" t="inlineStr"/>
+      <c r="K167" s="3" t="inlineStr"/>
+      <c r="L167" s="3" t="inlineStr"/>
+      <c r="M167" s="3" t="inlineStr"/>
+      <c r="N167" s="3" t="inlineStr"/>
     </row>
     <row r="168" ht="18" customHeight="1">
       <c r="A168" s="3" t="inlineStr"/>
@@ -2460,6 +3370,11 @@
       <c r="G168" s="3" t="inlineStr"/>
       <c r="H168" s="3" t="inlineStr"/>
       <c r="I168" s="3" t="inlineStr"/>
+      <c r="J168" s="3" t="inlineStr"/>
+      <c r="K168" s="3" t="inlineStr"/>
+      <c r="L168" s="3" t="inlineStr"/>
+      <c r="M168" s="3" t="inlineStr"/>
+      <c r="N168" s="3" t="inlineStr"/>
     </row>
     <row r="169" ht="18" customHeight="1">
       <c r="A169" s="3" t="inlineStr"/>
@@ -2471,6 +3386,11 @@
       <c r="G169" s="3" t="inlineStr"/>
       <c r="H169" s="3" t="inlineStr"/>
       <c r="I169" s="3" t="inlineStr"/>
+      <c r="J169" s="3" t="inlineStr"/>
+      <c r="K169" s="3" t="inlineStr"/>
+      <c r="L169" s="3" t="inlineStr"/>
+      <c r="M169" s="3" t="inlineStr"/>
+      <c r="N169" s="3" t="inlineStr"/>
     </row>
     <row r="170" ht="18" customHeight="1">
       <c r="A170" s="3" t="inlineStr"/>
@@ -2482,6 +3402,11 @@
       <c r="G170" s="3" t="inlineStr"/>
       <c r="H170" s="3" t="inlineStr"/>
       <c r="I170" s="3" t="inlineStr"/>
+      <c r="J170" s="3" t="inlineStr"/>
+      <c r="K170" s="3" t="inlineStr"/>
+      <c r="L170" s="3" t="inlineStr"/>
+      <c r="M170" s="3" t="inlineStr"/>
+      <c r="N170" s="3" t="inlineStr"/>
     </row>
     <row r="171" ht="18" customHeight="1">
       <c r="A171" s="3" t="inlineStr"/>
@@ -2493,6 +3418,11 @@
       <c r="G171" s="3" t="inlineStr"/>
       <c r="H171" s="3" t="inlineStr"/>
       <c r="I171" s="3" t="inlineStr"/>
+      <c r="J171" s="3" t="inlineStr"/>
+      <c r="K171" s="3" t="inlineStr"/>
+      <c r="L171" s="3" t="inlineStr"/>
+      <c r="M171" s="3" t="inlineStr"/>
+      <c r="N171" s="3" t="inlineStr"/>
     </row>
     <row r="172" ht="18" customHeight="1">
       <c r="A172" s="3" t="inlineStr"/>
@@ -2504,6 +3434,11 @@
       <c r="G172" s="3" t="inlineStr"/>
       <c r="H172" s="3" t="inlineStr"/>
       <c r="I172" s="3" t="inlineStr"/>
+      <c r="J172" s="3" t="inlineStr"/>
+      <c r="K172" s="3" t="inlineStr"/>
+      <c r="L172" s="3" t="inlineStr"/>
+      <c r="M172" s="3" t="inlineStr"/>
+      <c r="N172" s="3" t="inlineStr"/>
     </row>
     <row r="173" ht="18" customHeight="1">
       <c r="A173" s="3" t="inlineStr"/>
@@ -2515,6 +3450,11 @@
       <c r="G173" s="3" t="inlineStr"/>
       <c r="H173" s="3" t="inlineStr"/>
       <c r="I173" s="3" t="inlineStr"/>
+      <c r="J173" s="3" t="inlineStr"/>
+      <c r="K173" s="3" t="inlineStr"/>
+      <c r="L173" s="3" t="inlineStr"/>
+      <c r="M173" s="3" t="inlineStr"/>
+      <c r="N173" s="3" t="inlineStr"/>
     </row>
     <row r="174" ht="18" customHeight="1">
       <c r="A174" s="3" t="inlineStr"/>
@@ -2526,6 +3466,11 @@
       <c r="G174" s="3" t="inlineStr"/>
       <c r="H174" s="3" t="inlineStr"/>
       <c r="I174" s="3" t="inlineStr"/>
+      <c r="J174" s="3" t="inlineStr"/>
+      <c r="K174" s="3" t="inlineStr"/>
+      <c r="L174" s="3" t="inlineStr"/>
+      <c r="M174" s="3" t="inlineStr"/>
+      <c r="N174" s="3" t="inlineStr"/>
     </row>
     <row r="175" ht="18" customHeight="1">
       <c r="A175" s="3" t="inlineStr"/>
@@ -2537,6 +3482,11 @@
       <c r="G175" s="3" t="inlineStr"/>
       <c r="H175" s="3" t="inlineStr"/>
       <c r="I175" s="3" t="inlineStr"/>
+      <c r="J175" s="3" t="inlineStr"/>
+      <c r="K175" s="3" t="inlineStr"/>
+      <c r="L175" s="3" t="inlineStr"/>
+      <c r="M175" s="3" t="inlineStr"/>
+      <c r="N175" s="3" t="inlineStr"/>
     </row>
     <row r="176" ht="18" customHeight="1">
       <c r="A176" s="3" t="inlineStr"/>
@@ -2548,6 +3498,11 @@
       <c r="G176" s="3" t="inlineStr"/>
       <c r="H176" s="3" t="inlineStr"/>
       <c r="I176" s="3" t="inlineStr"/>
+      <c r="J176" s="3" t="inlineStr"/>
+      <c r="K176" s="3" t="inlineStr"/>
+      <c r="L176" s="3" t="inlineStr"/>
+      <c r="M176" s="3" t="inlineStr"/>
+      <c r="N176" s="3" t="inlineStr"/>
     </row>
     <row r="177" ht="18" customHeight="1">
       <c r="A177" s="3" t="inlineStr"/>
@@ -2559,6 +3514,11 @@
       <c r="G177" s="3" t="inlineStr"/>
       <c r="H177" s="3" t="inlineStr"/>
       <c r="I177" s="3" t="inlineStr"/>
+      <c r="J177" s="3" t="inlineStr"/>
+      <c r="K177" s="3" t="inlineStr"/>
+      <c r="L177" s="3" t="inlineStr"/>
+      <c r="M177" s="3" t="inlineStr"/>
+      <c r="N177" s="3" t="inlineStr"/>
     </row>
     <row r="178" ht="18" customHeight="1">
       <c r="A178" s="3" t="inlineStr"/>
@@ -2570,6 +3530,11 @@
       <c r="G178" s="3" t="inlineStr"/>
       <c r="H178" s="3" t="inlineStr"/>
       <c r="I178" s="3" t="inlineStr"/>
+      <c r="J178" s="3" t="inlineStr"/>
+      <c r="K178" s="3" t="inlineStr"/>
+      <c r="L178" s="3" t="inlineStr"/>
+      <c r="M178" s="3" t="inlineStr"/>
+      <c r="N178" s="3" t="inlineStr"/>
     </row>
     <row r="179" ht="18" customHeight="1">
       <c r="A179" s="3" t="inlineStr"/>
@@ -2581,6 +3546,11 @@
       <c r="G179" s="3" t="inlineStr"/>
       <c r="H179" s="3" t="inlineStr"/>
       <c r="I179" s="3" t="inlineStr"/>
+      <c r="J179" s="3" t="inlineStr"/>
+      <c r="K179" s="3" t="inlineStr"/>
+      <c r="L179" s="3" t="inlineStr"/>
+      <c r="M179" s="3" t="inlineStr"/>
+      <c r="N179" s="3" t="inlineStr"/>
     </row>
     <row r="180" ht="18" customHeight="1">
       <c r="A180" s="3" t="inlineStr"/>
@@ -2592,6 +3562,11 @@
       <c r="G180" s="3" t="inlineStr"/>
       <c r="H180" s="3" t="inlineStr"/>
       <c r="I180" s="3" t="inlineStr"/>
+      <c r="J180" s="3" t="inlineStr"/>
+      <c r="K180" s="3" t="inlineStr"/>
+      <c r="L180" s="3" t="inlineStr"/>
+      <c r="M180" s="3" t="inlineStr"/>
+      <c r="N180" s="3" t="inlineStr"/>
     </row>
     <row r="181" ht="18" customHeight="1">
       <c r="A181" s="3" t="inlineStr"/>
@@ -2603,6 +3578,11 @@
       <c r="G181" s="3" t="inlineStr"/>
       <c r="H181" s="3" t="inlineStr"/>
       <c r="I181" s="3" t="inlineStr"/>
+      <c r="J181" s="3" t="inlineStr"/>
+      <c r="K181" s="3" t="inlineStr"/>
+      <c r="L181" s="3" t="inlineStr"/>
+      <c r="M181" s="3" t="inlineStr"/>
+      <c r="N181" s="3" t="inlineStr"/>
     </row>
     <row r="182" ht="18" customHeight="1">
       <c r="A182" s="3" t="inlineStr"/>
@@ -2614,6 +3594,11 @@
       <c r="G182" s="3" t="inlineStr"/>
       <c r="H182" s="3" t="inlineStr"/>
       <c r="I182" s="3" t="inlineStr"/>
+      <c r="J182" s="3" t="inlineStr"/>
+      <c r="K182" s="3" t="inlineStr"/>
+      <c r="L182" s="3" t="inlineStr"/>
+      <c r="M182" s="3" t="inlineStr"/>
+      <c r="N182" s="3" t="inlineStr"/>
     </row>
     <row r="183" ht="18" customHeight="1">
       <c r="A183" s="3" t="inlineStr"/>
@@ -2625,6 +3610,11 @@
       <c r="G183" s="3" t="inlineStr"/>
       <c r="H183" s="3" t="inlineStr"/>
       <c r="I183" s="3" t="inlineStr"/>
+      <c r="J183" s="3" t="inlineStr"/>
+      <c r="K183" s="3" t="inlineStr"/>
+      <c r="L183" s="3" t="inlineStr"/>
+      <c r="M183" s="3" t="inlineStr"/>
+      <c r="N183" s="3" t="inlineStr"/>
     </row>
     <row r="184" ht="18" customHeight="1">
       <c r="A184" s="3" t="inlineStr"/>
@@ -2636,6 +3626,11 @@
       <c r="G184" s="3" t="inlineStr"/>
       <c r="H184" s="3" t="inlineStr"/>
       <c r="I184" s="3" t="inlineStr"/>
+      <c r="J184" s="3" t="inlineStr"/>
+      <c r="K184" s="3" t="inlineStr"/>
+      <c r="L184" s="3" t="inlineStr"/>
+      <c r="M184" s="3" t="inlineStr"/>
+      <c r="N184" s="3" t="inlineStr"/>
     </row>
     <row r="185" ht="18" customHeight="1">
       <c r="A185" s="3" t="inlineStr"/>
@@ -2647,6 +3642,11 @@
       <c r="G185" s="3" t="inlineStr"/>
       <c r="H185" s="3" t="inlineStr"/>
       <c r="I185" s="3" t="inlineStr"/>
+      <c r="J185" s="3" t="inlineStr"/>
+      <c r="K185" s="3" t="inlineStr"/>
+      <c r="L185" s="3" t="inlineStr"/>
+      <c r="M185" s="3" t="inlineStr"/>
+      <c r="N185" s="3" t="inlineStr"/>
     </row>
     <row r="186" ht="18" customHeight="1">
       <c r="A186" s="3" t="inlineStr"/>
@@ -2658,6 +3658,11 @@
       <c r="G186" s="3" t="inlineStr"/>
       <c r="H186" s="3" t="inlineStr"/>
       <c r="I186" s="3" t="inlineStr"/>
+      <c r="J186" s="3" t="inlineStr"/>
+      <c r="K186" s="3" t="inlineStr"/>
+      <c r="L186" s="3" t="inlineStr"/>
+      <c r="M186" s="3" t="inlineStr"/>
+      <c r="N186" s="3" t="inlineStr"/>
     </row>
     <row r="187" ht="18" customHeight="1">
       <c r="A187" s="3" t="inlineStr"/>
@@ -2669,6 +3674,11 @@
       <c r="G187" s="3" t="inlineStr"/>
       <c r="H187" s="3" t="inlineStr"/>
       <c r="I187" s="3" t="inlineStr"/>
+      <c r="J187" s="3" t="inlineStr"/>
+      <c r="K187" s="3" t="inlineStr"/>
+      <c r="L187" s="3" t="inlineStr"/>
+      <c r="M187" s="3" t="inlineStr"/>
+      <c r="N187" s="3" t="inlineStr"/>
     </row>
     <row r="188" ht="18" customHeight="1">
       <c r="A188" s="3" t="inlineStr"/>
@@ -2680,6 +3690,11 @@
       <c r="G188" s="3" t="inlineStr"/>
       <c r="H188" s="3" t="inlineStr"/>
       <c r="I188" s="3" t="inlineStr"/>
+      <c r="J188" s="3" t="inlineStr"/>
+      <c r="K188" s="3" t="inlineStr"/>
+      <c r="L188" s="3" t="inlineStr"/>
+      <c r="M188" s="3" t="inlineStr"/>
+      <c r="N188" s="3" t="inlineStr"/>
     </row>
     <row r="189" ht="18" customHeight="1">
       <c r="A189" s="3" t="inlineStr"/>
@@ -2691,6 +3706,11 @@
       <c r="G189" s="3" t="inlineStr"/>
       <c r="H189" s="3" t="inlineStr"/>
       <c r="I189" s="3" t="inlineStr"/>
+      <c r="J189" s="3" t="inlineStr"/>
+      <c r="K189" s="3" t="inlineStr"/>
+      <c r="L189" s="3" t="inlineStr"/>
+      <c r="M189" s="3" t="inlineStr"/>
+      <c r="N189" s="3" t="inlineStr"/>
     </row>
     <row r="190" ht="18" customHeight="1">
       <c r="A190" s="3" t="inlineStr"/>
@@ -2702,6 +3722,11 @@
       <c r="G190" s="3" t="inlineStr"/>
       <c r="H190" s="3" t="inlineStr"/>
       <c r="I190" s="3" t="inlineStr"/>
+      <c r="J190" s="3" t="inlineStr"/>
+      <c r="K190" s="3" t="inlineStr"/>
+      <c r="L190" s="3" t="inlineStr"/>
+      <c r="M190" s="3" t="inlineStr"/>
+      <c r="N190" s="3" t="inlineStr"/>
     </row>
     <row r="191" ht="18" customHeight="1">
       <c r="A191" s="3" t="inlineStr"/>
@@ -2713,6 +3738,11 @@
       <c r="G191" s="3" t="inlineStr"/>
       <c r="H191" s="3" t="inlineStr"/>
       <c r="I191" s="3" t="inlineStr"/>
+      <c r="J191" s="3" t="inlineStr"/>
+      <c r="K191" s="3" t="inlineStr"/>
+      <c r="L191" s="3" t="inlineStr"/>
+      <c r="M191" s="3" t="inlineStr"/>
+      <c r="N191" s="3" t="inlineStr"/>
     </row>
     <row r="192" ht="18" customHeight="1">
       <c r="A192" s="3" t="inlineStr"/>
@@ -2724,6 +3754,11 @@
       <c r="G192" s="3" t="inlineStr"/>
       <c r="H192" s="3" t="inlineStr"/>
       <c r="I192" s="3" t="inlineStr"/>
+      <c r="J192" s="3" t="inlineStr"/>
+      <c r="K192" s="3" t="inlineStr"/>
+      <c r="L192" s="3" t="inlineStr"/>
+      <c r="M192" s="3" t="inlineStr"/>
+      <c r="N192" s="3" t="inlineStr"/>
     </row>
     <row r="193" ht="18" customHeight="1">
       <c r="A193" s="3" t="inlineStr"/>
@@ -2735,6 +3770,11 @@
       <c r="G193" s="3" t="inlineStr"/>
       <c r="H193" s="3" t="inlineStr"/>
       <c r="I193" s="3" t="inlineStr"/>
+      <c r="J193" s="3" t="inlineStr"/>
+      <c r="K193" s="3" t="inlineStr"/>
+      <c r="L193" s="3" t="inlineStr"/>
+      <c r="M193" s="3" t="inlineStr"/>
+      <c r="N193" s="3" t="inlineStr"/>
     </row>
     <row r="194" ht="18" customHeight="1">
       <c r="A194" s="3" t="inlineStr"/>
@@ -2746,6 +3786,11 @@
       <c r="G194" s="3" t="inlineStr"/>
       <c r="H194" s="3" t="inlineStr"/>
       <c r="I194" s="3" t="inlineStr"/>
+      <c r="J194" s="3" t="inlineStr"/>
+      <c r="K194" s="3" t="inlineStr"/>
+      <c r="L194" s="3" t="inlineStr"/>
+      <c r="M194" s="3" t="inlineStr"/>
+      <c r="N194" s="3" t="inlineStr"/>
     </row>
     <row r="195" ht="18" customHeight="1">
       <c r="A195" s="3" t="inlineStr"/>
@@ -2757,6 +3802,11 @@
       <c r="G195" s="3" t="inlineStr"/>
       <c r="H195" s="3" t="inlineStr"/>
       <c r="I195" s="3" t="inlineStr"/>
+      <c r="J195" s="3" t="inlineStr"/>
+      <c r="K195" s="3" t="inlineStr"/>
+      <c r="L195" s="3" t="inlineStr"/>
+      <c r="M195" s="3" t="inlineStr"/>
+      <c r="N195" s="3" t="inlineStr"/>
     </row>
     <row r="196" ht="18" customHeight="1">
       <c r="A196" s="3" t="inlineStr"/>
@@ -2768,6 +3818,11 @@
       <c r="G196" s="3" t="inlineStr"/>
       <c r="H196" s="3" t="inlineStr"/>
       <c r="I196" s="3" t="inlineStr"/>
+      <c r="J196" s="3" t="inlineStr"/>
+      <c r="K196" s="3" t="inlineStr"/>
+      <c r="L196" s="3" t="inlineStr"/>
+      <c r="M196" s="3" t="inlineStr"/>
+      <c r="N196" s="3" t="inlineStr"/>
     </row>
     <row r="197" ht="18" customHeight="1">
       <c r="A197" s="3" t="inlineStr"/>
@@ -2779,6 +3834,11 @@
       <c r="G197" s="3" t="inlineStr"/>
       <c r="H197" s="3" t="inlineStr"/>
       <c r="I197" s="3" t="inlineStr"/>
+      <c r="J197" s="3" t="inlineStr"/>
+      <c r="K197" s="3" t="inlineStr"/>
+      <c r="L197" s="3" t="inlineStr"/>
+      <c r="M197" s="3" t="inlineStr"/>
+      <c r="N197" s="3" t="inlineStr"/>
     </row>
     <row r="198" ht="18" customHeight="1">
       <c r="A198" s="3" t="inlineStr"/>
@@ -2790,6 +3850,11 @@
       <c r="G198" s="3" t="inlineStr"/>
       <c r="H198" s="3" t="inlineStr"/>
       <c r="I198" s="3" t="inlineStr"/>
+      <c r="J198" s="3" t="inlineStr"/>
+      <c r="K198" s="3" t="inlineStr"/>
+      <c r="L198" s="3" t="inlineStr"/>
+      <c r="M198" s="3" t="inlineStr"/>
+      <c r="N198" s="3" t="inlineStr"/>
     </row>
     <row r="199" ht="18" customHeight="1">
       <c r="A199" s="3" t="inlineStr"/>
@@ -2801,6 +3866,11 @@
       <c r="G199" s="3" t="inlineStr"/>
       <c r="H199" s="3" t="inlineStr"/>
       <c r="I199" s="3" t="inlineStr"/>
+      <c r="J199" s="3" t="inlineStr"/>
+      <c r="K199" s="3" t="inlineStr"/>
+      <c r="L199" s="3" t="inlineStr"/>
+      <c r="M199" s="3" t="inlineStr"/>
+      <c r="N199" s="3" t="inlineStr"/>
     </row>
     <row r="200" ht="18" customHeight="1">
       <c r="A200" s="3" t="inlineStr"/>
@@ -2812,6 +3882,11 @@
       <c r="G200" s="3" t="inlineStr"/>
       <c r="H200" s="3" t="inlineStr"/>
       <c r="I200" s="3" t="inlineStr"/>
+      <c r="J200" s="3" t="inlineStr"/>
+      <c r="K200" s="3" t="inlineStr"/>
+      <c r="L200" s="3" t="inlineStr"/>
+      <c r="M200" s="3" t="inlineStr"/>
+      <c r="N200" s="3" t="inlineStr"/>
     </row>
     <row r="201" ht="18" customHeight="1">
       <c r="A201" s="3" t="inlineStr"/>
@@ -2823,6 +3898,11 @@
       <c r="G201" s="3" t="inlineStr"/>
       <c r="H201" s="3" t="inlineStr"/>
       <c r="I201" s="3" t="inlineStr"/>
+      <c r="J201" s="3" t="inlineStr"/>
+      <c r="K201" s="3" t="inlineStr"/>
+      <c r="L201" s="3" t="inlineStr"/>
+      <c r="M201" s="3" t="inlineStr"/>
+      <c r="N201" s="3" t="inlineStr"/>
     </row>
     <row r="202" ht="18" customHeight="1">
       <c r="A202" s="3" t="inlineStr"/>
@@ -2834,6 +3914,11 @@
       <c r="G202" s="3" t="inlineStr"/>
       <c r="H202" s="3" t="inlineStr"/>
       <c r="I202" s="3" t="inlineStr"/>
+      <c r="J202" s="3" t="inlineStr"/>
+      <c r="K202" s="3" t="inlineStr"/>
+      <c r="L202" s="3" t="inlineStr"/>
+      <c r="M202" s="3" t="inlineStr"/>
+      <c r="N202" s="3" t="inlineStr"/>
     </row>
     <row r="203" ht="18" customHeight="1">
       <c r="A203" s="3" t="inlineStr"/>
@@ -2845,6 +3930,11 @@
       <c r="G203" s="3" t="inlineStr"/>
       <c r="H203" s="3" t="inlineStr"/>
       <c r="I203" s="3" t="inlineStr"/>
+      <c r="J203" s="3" t="inlineStr"/>
+      <c r="K203" s="3" t="inlineStr"/>
+      <c r="L203" s="3" t="inlineStr"/>
+      <c r="M203" s="3" t="inlineStr"/>
+      <c r="N203" s="3" t="inlineStr"/>
     </row>
     <row r="204" ht="18" customHeight="1">
       <c r="A204" s="3" t="inlineStr"/>
@@ -2856,6 +3946,11 @@
       <c r="G204" s="3" t="inlineStr"/>
       <c r="H204" s="3" t="inlineStr"/>
       <c r="I204" s="3" t="inlineStr"/>
+      <c r="J204" s="3" t="inlineStr"/>
+      <c r="K204" s="3" t="inlineStr"/>
+      <c r="L204" s="3" t="inlineStr"/>
+      <c r="M204" s="3" t="inlineStr"/>
+      <c r="N204" s="3" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2868,11 +3963,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B15"/>
+  <dimension ref="A1:B19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
-    <col width="50" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="55" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2881,169 +3976,217 @@
           <t>ALAN</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="5" t="inlineStr">
         <is>
           <t>AÇIKLAMA</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="5" t="inlineStr">
-        <is>
-          <t>Ad *</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
+      <c r="A2" s="6" t="inlineStr">
+        <is>
+          <t>S.NO</t>
+        </is>
+      </c>
+      <c r="B2" s="5" t="inlineStr">
+        <is>
+          <t>Sıra numarası — otomatik doldurabilirsiniz</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="6" t="inlineStr">
+        <is>
+          <t>ADI *</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
         <is>
           <t>Öğrencinin adı (zorunlu)</t>
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="5" t="inlineStr">
-        <is>
-          <t>Soyad *</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
+    <row r="4">
+      <c r="A4" s="6" t="inlineStr">
+        <is>
+          <t>SOYADI *</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
         <is>
           <t>Öğrencinin soyadı (zorunlu)</t>
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="5" t="inlineStr">
-        <is>
-          <t>Doğum Tarihi</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
+    <row r="5">
+      <c r="A5" s="6" t="inlineStr">
+        <is>
+          <t>TC NO</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>11 haneli TC kimlik numarası</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="6" t="inlineStr">
+        <is>
+          <t>DOĞUM TARİHİ</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
         <is>
           <t>YYYY-AA-GG formatında. Örnek: 2015-03-15</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="5" t="inlineStr">
-        <is>
-          <t>Cinsiyet *</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>kiz veya erkek yazın (küçük harf) (zorunlu)</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="5" t="inlineStr">
-        <is>
-          <t>Veli Adı Soyadı *</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Velinin tam adı (zorunlu)</t>
-        </is>
-      </c>
-    </row>
     <row r="7">
-      <c r="A7" s="5" t="inlineStr">
-        <is>
-          <t>Veli Telefonu *</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
+      <c r="A7" s="6" t="inlineStr">
+        <is>
+          <t>CİNSİYET *</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>kiz veya erkek yazın (zorunlu)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="6" t="inlineStr">
+        <is>
+          <t>YAŞI</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>Rakam olarak. Örnek: 11</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="6" t="inlineStr">
+        <is>
+          <t>ADRES</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>Öğrencinin adresi</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="6" t="inlineStr">
+        <is>
+          <t>VELİ ADI *</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>Velinin adı (zorunlu)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="6" t="inlineStr">
+        <is>
+          <t>VELİ SOYADI *</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>Velinin soyadı (zorunlu)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="6" t="inlineStr">
+        <is>
+          <t>VELİ ADRESİ</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>Velinin adresi</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="6" t="inlineStr">
+        <is>
+          <t>GSM NUMARASI *</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
         <is>
           <t>05xxxxxxxxx formatında (zorunlu)</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="5" t="inlineStr">
-        <is>
-          <t>Mahalle</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>Öğrencinin mahallesi (opsiyonel)</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="5" t="inlineStr">
-        <is>
-          <t>TC Kimlik No</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>11 haneli TC no (opsiyonel)</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="5" t="inlineStr">
-        <is>
-          <t>Sınıf Adı</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
+    <row r="14">
+      <c r="A14" s="6" t="inlineStr">
+        <is>
+          <t>KAYIT TARİHİ</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>YYYY-AA-GG formatında. Boş bırakılırsa bugün kullanılır</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="6" t="inlineStr">
+        <is>
+          <t>SINIF</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
         <is>
           <t>Sistemdeki sınıf adıyla aynı olmalı (opsiyonel)</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="5" t="inlineStr"/>
-      <c r="B11" t="inlineStr"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="5" t="inlineStr">
+    <row r="16">
+      <c r="A16" s="6" t="inlineStr"/>
+      <c r="B16" s="5" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="6" t="inlineStr">
         <is>
           <t>NOT</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
+      <c r="B17" s="5" t="inlineStr">
         <is>
           <t>* işaretli alanlar zorunludur</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="5" t="inlineStr">
+    <row r="18">
+      <c r="A18" s="6" t="inlineStr">
         <is>
           <t>NOT</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>Yeşil satırlar örnek veridir, silebilirsiniz</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="5" t="inlineStr">
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>Yeşil satırlar örnek verilerdir — silebilirsiniz</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="6" t="inlineStr">
         <is>
           <t>NOT</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr">
+      <c r="B19" s="5" t="inlineStr">
         <is>
           <t>En fazla 200 öğrenci yükleyebilirsiniz</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="5" t="inlineStr">
-        <is>
-          <t>NOT</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>Telefon başında 0 olmalı: 05xxxxxxxxx</t>
         </is>
       </c>
     </row>

</xml_diff>